<commit_message>
data renew in Mar. 2026
</commit_message>
<xml_diff>
--- a/abx.xlsx
+++ b/abx.xlsx
@@ -1,21 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="ATC" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Sheet2" sheetId="3" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ATC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Sheet1!$A$1:$F$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$148</definedName>
   </definedNames>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="695">
   <si>
     <t>drug_id</t>
   </si>
@@ -38,10 +45,10 @@
     <t>PER02E</t>
   </si>
   <si>
-    <t>Periocline Periodontal Oint</t>
-  </si>
-  <si>
-    <t>Minocycline(Periocline) Periodontal Oint</t>
+    <t xml:space="preserve">Periocline Periodontal Oint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minocycline(Periocline) Periodontal Oint</t>
   </si>
   <si>
     <t>A01AB23</t>
@@ -50,10 +57,10 @@
     <t>MYC01S</t>
   </si>
   <si>
-    <t>Mycostatin Susp 2400000 Units/24ml</t>
-  </si>
-  <si>
-    <t>Nystatin(Mycostatin) Susp 2400000 Units/24ml</t>
+    <t xml:space="preserve">Mycostatin Susp 2400000 Units/24ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nystatin(Mycostatin) Susp 2400000 Units/24ml</t>
   </si>
   <si>
     <t>A07AA02</t>
@@ -62,19 +69,19 @@
     <t>NYS01O</t>
   </si>
   <si>
-    <t>Nystatin 500000u Cap</t>
-  </si>
-  <si>
-    <t>PK: poorly abs</t>
+    <t xml:space="preserve">Nystatin 500000u Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PK: poorly abs</t>
   </si>
   <si>
     <t>HUM01O</t>
   </si>
   <si>
-    <t>Humatin 250mg Cap  (公費)</t>
-  </si>
-  <si>
-    <t>Paromomycin (Humatin) 250mg Cap (公費)</t>
+    <t xml:space="preserve">Humatin 250mg Cap  (公費)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paromomycin (Humatin) 250mg Cap (公費)</t>
   </si>
   <si>
     <t>A07AA06</t>
@@ -83,10 +90,10 @@
     <t>DIF02O</t>
   </si>
   <si>
-    <t>Dificid 200mg Tab#</t>
-  </si>
-  <si>
-    <t>Fidaxomicin (Dificid) 200mg Tab</t>
+    <t xml:space="preserve">Dificid 200mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fidaxomicin (Dificid) 200mg Tab</t>
   </si>
   <si>
     <t>A07AA12</t>
@@ -95,10 +102,10 @@
     <t>CAM05O</t>
   </si>
   <si>
-    <t>Camisan 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Terbinafine(Camisan) 250mg Tab#</t>
+    <t xml:space="preserve">Camisan 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terbinafine(Camisan) 250mg Tab#</t>
   </si>
   <si>
     <t>D01BA02</t>
@@ -107,19 +114,19 @@
     <t>LAM01O</t>
   </si>
   <si>
-    <t>Lamisil 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Terbinafine(Lamisil) 250mg Tab#</t>
+    <t xml:space="preserve">Lamisil 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terbinafine(Lamisil) 250mg Tab#</t>
   </si>
   <si>
     <t>DOX02O</t>
   </si>
   <si>
-    <t>Doxymycin 100mg Ec Cap</t>
-  </si>
-  <si>
-    <t>Doxycycline(Doxymycin) 100mg EC Cap</t>
+    <t xml:space="preserve">Doxymycin 100mg Ec Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doxycycline(Doxymycin) 100mg EC Cap</t>
   </si>
   <si>
     <t>J01AA02</t>
@@ -131,22 +138,22 @@
     <t>TET02O</t>
   </si>
   <si>
-    <t>Tetracycline HCl 250mg Cap</t>
+    <t xml:space="preserve">Tetracycline HCl 250mg Cap</t>
   </si>
   <si>
     <t>J01AA07</t>
   </si>
   <si>
-    <t>建議量: 500 mg q6h@ renal dysfunction: 建議選用doxy</t>
+    <t xml:space="preserve">建議量: 500 mg q6h@ renal dysfunction: 建議選用doxy</t>
   </si>
   <si>
     <t>CYC01O</t>
   </si>
   <si>
-    <t>Cyclin 100mg Cap</t>
-  </si>
-  <si>
-    <t>Minocycline(Cyclin) 100mg Cap</t>
+    <t xml:space="preserve">Cyclin 100mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minocycline(Cyclin) 100mg Cap</t>
   </si>
   <si>
     <t>J01AA08</t>
@@ -155,157 +162,157 @@
     <t>MEN01I</t>
   </si>
   <si>
-    <t>Menocik 100mg Vial</t>
-  </si>
-  <si>
-    <t>Minocycline(Menocik) 100mg Vial</t>
-  </si>
-  <si>
-    <t>100 mg q12h drip 1hr@ lipophillic</t>
+    <t xml:space="preserve">Menocik 100mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minocycline(Menocik) 100mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 mg q12h drip 1hr@ lipophillic</t>
   </si>
   <si>
     <t>MER02O</t>
   </si>
   <si>
-    <t>Mero 100mg Cap</t>
-  </si>
-  <si>
-    <t>Minocycline (Mero) 100mg Cap</t>
-  </si>
-  <si>
-    <t>建議量: 100 mg q12h</t>
+    <t xml:space="preserve">Mero 100mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minocycline (Mero) 100mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量: 100 mg q12h</t>
   </si>
   <si>
     <t>TIG01I</t>
   </si>
   <si>
-    <t>Tigelin 50mg Vial</t>
-  </si>
-  <si>
-    <t>Tigecycline(Tigelin) 50mg Vial</t>
+    <t xml:space="preserve">Tigelin 50mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tigecycline(Tigelin) 50mg Vial</t>
   </si>
   <si>
     <t>J01AA12</t>
   </si>
   <si>
-    <t>mino衍生@ age over than 8 years old</t>
+    <t xml:space="preserve">mino衍生@ age over than 8 years old</t>
   </si>
   <si>
     <t>TYG01I</t>
   </si>
   <si>
-    <t>Tygacil 50mg Vial#</t>
-  </si>
-  <si>
-    <t>Tigecycline(Tygacil) 50mg Vial#</t>
+    <t xml:space="preserve">Tygacil 50mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tigecycline(Tygacil) 50mg Vial#</t>
   </si>
   <si>
     <t>AMP01O</t>
   </si>
   <si>
-    <t>Ampicillin 500mg Cap</t>
-  </si>
-  <si>
-    <t>Ampicillin(Ampicillin) 500mg Cap</t>
+    <t xml:space="preserve">Ampicillin 500mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ampicillin(Ampicillin) 500mg Cap</t>
   </si>
   <si>
     <t>J01CA01</t>
   </si>
   <si>
-    <t>小兒: 100 to 300 mg per kg per day 分 q4h to q6h@ Ccr less 30: 1 to 2 gm q8h@ Ccr less 10 or HD: altered to q12h</t>
+    <t xml:space="preserve">小兒: 100 to 300 mg per kg per day 分 q4h to q6h@ Ccr less 30: 1 to 2 gm q8h@ Ccr less 10 or HD: altered to q12h</t>
   </si>
   <si>
     <t>AMP03I</t>
   </si>
   <si>
-    <t>Ampolin 500mg Vial</t>
-  </si>
-  <si>
-    <t>Ampicillin(Ampolin) 500mg Vial</t>
+    <t xml:space="preserve">Ampolin 500mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ampicillin(Ampolin) 500mg Vial</t>
   </si>
   <si>
     <t>SER03I</t>
   </si>
   <si>
-    <t>Servicillin 500mg Vial</t>
-  </si>
-  <si>
-    <t>Ampicillin(Servicillin) 500mg Vial</t>
+    <t xml:space="preserve">Servicillin 500mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ampicillin(Servicillin) 500mg Vial</t>
   </si>
   <si>
     <t>AMO01I</t>
   </si>
   <si>
-    <t>AmoClav 1.2g Vial</t>
+    <t xml:space="preserve">AmoClav 1.2g Vial</t>
   </si>
   <si>
     <t>J01CA04</t>
   </si>
   <si>
-    <t>建議量:  1.2 gm q8h@ Ccr less 30: 1vial q12h@ Ccr less 10 or HD: 1 vial qd</t>
+    <t xml:space="preserve">建議量:  1.2 gm q8h@ Ccr less 30: 1vial q12h@ Ccr less 10 or HD: 1 vial qd</t>
   </si>
   <si>
     <t>AMO01O</t>
   </si>
   <si>
-    <t>Amoxicillin 250mg Cap YungShin</t>
+    <t xml:space="preserve">Amoxicillin 250mg Cap YungShin</t>
   </si>
   <si>
     <t>J01CA04O</t>
   </si>
   <si>
-    <t>建議量:  1 gm q8h@ Ccr less 30: 1 gm q12h@ Ccr less 10 or HD: 1 gm qd</t>
+    <t xml:space="preserve">建議量:  1 gm q8h@ Ccr less 30: 1 gm q12h@ Ccr less 10 or HD: 1 gm qd</t>
   </si>
   <si>
     <t>AMO02O</t>
   </si>
   <si>
-    <t>Amoxicillin 250mg Cap TBC</t>
+    <t xml:space="preserve">Amoxicillin 250mg Cap TBC</t>
   </si>
   <si>
     <t>AMO02S</t>
   </si>
   <si>
-    <t>Amolin Susp 25mg/ml;60ml#</t>
-  </si>
-  <si>
-    <t>Amoxicillin(Amolin) Susp 25mg/ml 60ml#</t>
+    <t xml:space="preserve">Amolin Susp 25mg/ml;60ml#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amoxicillin(Amolin) Susp 25mg/ml 60ml#</t>
   </si>
   <si>
     <t>J01CA04S</t>
   </si>
   <si>
-    <t>80 to 90 mg per kg per day for q8h to q12h</t>
+    <t xml:space="preserve">80 to 90 mg per kg per day for q8h to q12h</t>
   </si>
   <si>
     <t>AMO04S</t>
   </si>
   <si>
-    <t>AMOLIN SUSP 50MG/ML;60ML</t>
-  </si>
-  <si>
-    <t>Amoxicillin(AMOLIN) Susp 50mg/ml 60ml</t>
+    <t xml:space="preserve">AMOLIN SUSP 50MG/ML;60ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amoxicillin(AMOLIN) Susp 50mg/ml 60ml</t>
   </si>
   <si>
     <t>PEN05I</t>
   </si>
   <si>
-    <t>Penicillin G 3000000U Vial</t>
+    <t xml:space="preserve">Penicillin G 3000000U Vial</t>
   </si>
   <si>
     <t>J01CE01</t>
   </si>
   <si>
-    <t>建議量: 1 vial q4h@ Ccr less than 30: q8h@ Ccr less than 10, HD or PD: q12h</t>
+    <t xml:space="preserve">建議量: 1 vial q4h@ Ccr less than 30: q8h@ Ccr less than 10, HD or PD: q12h</t>
   </si>
   <si>
     <t>BIC03I</t>
   </si>
   <si>
-    <t>Bicillin L-A 2.4MIU/4ml Susp Inj</t>
-  </si>
-  <si>
-    <t>Penicillin G Benzathine (Bicillin) L-A 2.4MIU/4ml Inj Susp</t>
+    <t xml:space="preserve">Bicillin L-A 2.4MIU/4ml Susp Inj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penicillin G Benzathine (Bicillin) L-A 2.4MIU/4ml Inj Susp</t>
   </si>
   <si>
     <t>J01CE08</t>
@@ -314,37 +321,37 @@
     <t>DIC03O</t>
   </si>
   <si>
-    <t>Diclocin 250mg Cap</t>
-  </si>
-  <si>
-    <t>Dicloxacillin(Diclocin) 250mg Cap</t>
+    <t xml:space="preserve">Diclocin 250mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dicloxacillin(Diclocin) 250mg Cap</t>
   </si>
   <si>
     <t>J01CF01</t>
   </si>
   <si>
-    <t>建議量: 500 mg q6h@ 主要經肝臟排泄@ 以1st cephas代替減少其副作用</t>
+    <t xml:space="preserve">建議量: 500 mg q6h@ 主要經肝臟排泄@ 以1st cephas代替減少其副作用</t>
   </si>
   <si>
     <t>OXA03I</t>
   </si>
   <si>
-    <t>Oxacillin Powder for Injection  1gm Vial</t>
+    <t xml:space="preserve">Oxacillin Powder for Injection  1gm Vial</t>
   </si>
   <si>
     <t>J01CF04</t>
   </si>
   <si>
-    <t>建議量: 1 to 2 gm q4h@ 主要經肝臟排泄</t>
+    <t xml:space="preserve">建議量: 1 to 2 gm q4h@ 主要經肝臟排泄</t>
   </si>
   <si>
     <t>MAX03I</t>
   </si>
   <si>
-    <t>Maxtam 500mg Vial</t>
-  </si>
-  <si>
-    <t>Sulbactam(Maxtam) 500mg Vial</t>
+    <t xml:space="preserve">Maxtam 500mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sulbactam(Maxtam) 500mg Vial</t>
   </si>
   <si>
     <t>J01CG01</t>
@@ -353,34 +360,34 @@
     <t>SUL01I</t>
   </si>
   <si>
-    <t>Sulbactam 500 mg Vial</t>
-  </si>
-  <si>
-    <t>Sulbactam 500mg Vial</t>
+    <t xml:space="preserve">Sulbactam 500 mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sulbactam 500mg Vial</t>
   </si>
   <si>
     <t>SUB01I</t>
   </si>
   <si>
-    <t>Subacillin Inj 1.5gm Vial#</t>
+    <t xml:space="preserve">Subacillin Inj 1.5gm Vial#</t>
   </si>
   <si>
     <t>J01CR01</t>
   </si>
   <si>
-    <t>建議量:  1.5 gm to 3 gm q6h @ Ccr less 30: 3 gm q12h@ Ccr less 10 or HD: 3 gm qd</t>
+    <t xml:space="preserve">建議量:  1.5 gm to 3 gm q6h @ Ccr less 30: 3 gm q12h@ Ccr less 10 or HD: 3 gm qd</t>
   </si>
   <si>
     <t>UNA01I</t>
   </si>
   <si>
-    <t>Unasyn 1.5gm Vial#</t>
+    <t xml:space="preserve">Unasyn 1.5gm Vial#</t>
   </si>
   <si>
     <t>AUG03O</t>
   </si>
   <si>
-    <t>Augmentin 1g Tab#</t>
+    <t xml:space="preserve">Augmentin 1g Tab#</t>
   </si>
   <si>
     <t>J01CR02</t>
@@ -389,49 +396,49 @@
     <t>AUG04S</t>
   </si>
   <si>
-    <t>Augmentin Syrup 457mg/5ml;35ml#</t>
-  </si>
-  <si>
-    <t>Augmentin Syrup 457mg/5ml 35ml#</t>
+    <t xml:space="preserve">Augmentin Syrup 457mg/5ml;35ml#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Augmentin Syrup 457mg/5ml 35ml#</t>
   </si>
   <si>
     <t>J01CR02S</t>
   </si>
   <si>
-    <t>40 to 45 mg per kg q8h to q12h 以 amoxi 計@ 高劑量: 2倍量頻次不變</t>
+    <t xml:space="preserve">40 to 45 mg per kg q8h to q12h 以 amoxi 計@ 高劑量: 2倍量頻次不變</t>
   </si>
   <si>
     <t>CUR01I</t>
   </si>
   <si>
-    <t>Curam 1.2g Vial</t>
-  </si>
-  <si>
-    <t>Curam 1.2gm Vial</t>
-  </si>
-  <si>
-    <t>建議量:  1 vial q8h@ 小兒: 30 mg per kg q8h 以 amoxi 計@ Ccr less than 30: q12h@ Ccr less than 10, HD or PD: qd</t>
+    <t xml:space="preserve">Curam 1.2g Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curam 1.2gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量:  1 vial q8h@ 小兒: 30 mg per kg q8h 以 amoxi 計@ Ccr less than 30: q12h@ Ccr less than 10, HD or PD: qd</t>
   </si>
   <si>
     <t>CUR01O</t>
   </si>
   <si>
-    <t>Curam FC 1g Tab#</t>
+    <t xml:space="preserve">Curam FC 1g Tab#</t>
   </si>
   <si>
     <t>J01CR02O</t>
   </si>
   <si>
-    <t>建議量:  1tab q8h@ Ccr less 30 or HD: clavulanate 排除較 amox 快易造成治療失敗</t>
+    <t xml:space="preserve">建議量:  1tab q8h@ Ccr less 30 or HD: clavulanate 排除較 amox 快易造成治療失敗</t>
   </si>
   <si>
     <t>UNA01O</t>
   </si>
   <si>
-    <t>Unasyn 375mg Tab#</t>
-  </si>
-  <si>
-    <t>Sultamicillin (Unasyn) 375mg Tab#</t>
+    <t xml:space="preserve">Unasyn 375mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sultamicillin (Unasyn) 375mg Tab#</t>
   </si>
   <si>
     <t>J01CR04</t>
@@ -440,55 +447,55 @@
     <t>TAP01I</t>
   </si>
   <si>
-    <t>Tapimycin 4.5gm Vial#</t>
+    <t xml:space="preserve">Tapimycin 4.5gm Vial#</t>
   </si>
   <si>
     <t>J01CR05</t>
   </si>
   <si>
-    <t>建議量:  4.5 gm q8h @ Ccr less 20 or HD: 4.5 gm q12h</t>
+    <t xml:space="preserve">建議量:  4.5 gm q8h @ Ccr less 20 or HD: 4.5 gm q12h</t>
   </si>
   <si>
     <t>TAZ02I</t>
   </si>
   <si>
-    <t>Tazocin 2.25gm Vial#</t>
+    <t xml:space="preserve">Tazocin 2.25gm Vial#</t>
   </si>
   <si>
     <t>CEP05O</t>
   </si>
   <si>
-    <t>Cephalexin 500mg Cap</t>
+    <t xml:space="preserve">Cephalexin 500mg Cap</t>
   </si>
   <si>
     <t>J01DB01</t>
   </si>
   <si>
-    <t>建議量:  500 mg to 1 gm q6h@ Ccr less 30: 1 gm q8h or q12h@ Ccr less 10 or HD: 1 gm qd</t>
+    <t xml:space="preserve">建議量:  500 mg to 1 gm q6h@ Ccr less 30: 1 gm q8h or q12h@ Ccr less 10 or HD: 1 gm qd</t>
   </si>
   <si>
     <t>ULE01S</t>
   </si>
   <si>
-    <t>Ulexin Susp 25mg/ml;60ml Bot</t>
-  </si>
-  <si>
-    <t>Cephalexin(Ulexin) Susp 25mg/ml 60ml Bot</t>
+    <t xml:space="preserve">Ulexin Susp 25mg/ml;60ml Bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cephalexin(Ulexin) Susp 25mg/ml 60ml Bot</t>
   </si>
   <si>
     <t>J01DB01O</t>
   </si>
   <si>
-    <t>10 mg to 20 mg per kg q6h</t>
+    <t xml:space="preserve">10 mg to 20 mg per kg q6h</t>
   </si>
   <si>
     <t>CEF06I</t>
   </si>
   <si>
-    <t>Cefa 1gm Vial</t>
-  </si>
-  <si>
-    <t>Cefazolin(Cefa) 1gm Vial</t>
+    <t xml:space="preserve">Cefa 1gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefazolin(Cefa) 1gm Vial</t>
   </si>
   <si>
     <t>J01DB04</t>
@@ -497,34 +504,34 @@
     <t>STA01I</t>
   </si>
   <si>
-    <t>Stazolin 1gm Vial</t>
-  </si>
-  <si>
-    <t>Cefazolin(Stazolin) 1gm Vial</t>
-  </si>
-  <si>
-    <t>建議量:  2 g q8h才能達到PD@ Ccr less than 30: 2 gm q12h@ Ccr less than 10 or HD PD: 1 gm qd</t>
+    <t xml:space="preserve">Stazolin 1gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefazolin(Stazolin) 1gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量:  2 g q8h才能達到PD@ Ccr less than 30: 2 gm q12h@ Ccr less than 10 or HD PD: 1 gm qd</t>
   </si>
   <si>
     <t>CEF01O</t>
   </si>
   <si>
-    <t>Ceflour FC 250mg Tab</t>
-  </si>
-  <si>
-    <t>CEFUROXIME(Ceflour) 250mg Tab</t>
+    <t xml:space="preserve">Ceflour FC 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CEFUROXIME(Ceflour) 250mg Tab</t>
   </si>
   <si>
     <t>J01DC02O</t>
   </si>
   <si>
-    <t>建議量:  500 mg q12h@ Ccr less 30 or HD PD: 500 mg qd</t>
+    <t xml:space="preserve">建議量:  500 mg q12h@ Ccr less 30 or HD PD: 500 mg qd</t>
   </si>
   <si>
     <t>CEF07I</t>
   </si>
   <si>
-    <t>Cefuroxime 750mg Vial#</t>
+    <t xml:space="preserve">Cefuroxime 750mg Vial#</t>
   </si>
   <si>
     <t>J01DC02</t>
@@ -533,109 +540,109 @@
     <t>FUR02I</t>
   </si>
   <si>
-    <t>Furoxime 750mg Vial#</t>
-  </si>
-  <si>
-    <t>建議量:  1.5 gm q8h@ Ccr less 30: 1.5 g q12h@ Ccr less 10 or HD: 1.5 g qd</t>
+    <t xml:space="preserve">Furoxime 750mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量:  1.5 gm q8h@ Ccr less 30: 1.5 g q12h@ Ccr less 10 or HD: 1.5 g qd</t>
   </si>
   <si>
     <t>FLU11I</t>
   </si>
   <si>
-    <t>Flumarin 1gm Vial#</t>
-  </si>
-  <si>
-    <t>Flomoxef(Flumarin) 1gm Vial#</t>
+    <t xml:space="preserve">Flumarin 1gm Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flomoxef(Flumarin) 1gm Vial#</t>
   </si>
   <si>
     <t>J01DC14</t>
   </si>
   <si>
-    <t>建議量:  1 g to 2 gm q6h@ 2.5gen or 3rd cephas for ESBL@ Ccr less than 50: 1 gm q12h@ Ccr less 25 or HD: 1 g qd</t>
+    <t xml:space="preserve">建議量:  1 g to 2 gm q6h@ 2.5gen or 3rd cephas for ESBL@ Ccr less than 50: 1 gm q12h@ Ccr less 25 or HD: 1 g qd</t>
   </si>
   <si>
     <t>CLA01I</t>
   </si>
   <si>
-    <t>Claforan IV Inj 2gm Vial</t>
-  </si>
-  <si>
-    <t>Cefotaxime(Claforan) 2gm Vial</t>
+    <t xml:space="preserve">Claforan IV Inj 2gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefotaxime(Claforan) 2gm Vial</t>
   </si>
   <si>
     <t>J01DD01</t>
   </si>
   <si>
-    <t>建議量:  2 gm q6h@ 小兒: 40 mg per kg q6h to q4h Max: 2 gm q6h@ Ccr less than 50: 2 gm q8h@ Ccr less than 30: 2 gm q12h@ Ccr less than 10, HD or PD: 1 gm qd</t>
+    <t xml:space="preserve">建議量:  2 gm q6h@ 小兒: 40 mg per kg q6h to q4h Max: 2 gm q6h@ Ccr less than 50: 2 gm q8h@ Ccr less than 30: 2 gm q12h@ Ccr less than 10, HD or PD: 1 gm qd</t>
   </si>
   <si>
     <t>TAT02I</t>
   </si>
   <si>
-    <t>Tatumcef 1gm Vial#</t>
-  </si>
-  <si>
-    <t>Ceftazidime(Tatumcef) 1gm Vial#</t>
+    <t xml:space="preserve">Tatumcef 1gm Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceftazidime(Tatumcef) 1gm Vial#</t>
   </si>
   <si>
     <t>J01DD02</t>
   </si>
   <si>
-    <t>3ed cephas@ 經驗性應以ceftriaxone取代@ 經驗性 for GNB UTI@ 建議量:  2 gm q8h@ Ccr less 50: 2 g q12h@ Ccr less 30: 2 g qd@ Ccr less 10 or HD: 1 g qd</t>
+    <t xml:space="preserve">3ed cephas@ 經驗性應以ceftriaxone取代@ 經驗性 for GNB UTI@ 建議量:  2 gm q8h@ Ccr less 50: 2 g q12h@ Ccr less 30: 2 g qd@ Ccr less 10 or HD: 1 g qd</t>
   </si>
   <si>
     <t>TAT03I</t>
   </si>
   <si>
-    <t>TATUMCEF 2GM VIAL</t>
-  </si>
-  <si>
-    <t>Ceftazidime(TATUMCEF) 2GM VIAL</t>
+    <t xml:space="preserve">TATUMCEF 2GM VIAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceftazidime(TATUMCEF) 2GM VIAL</t>
   </si>
   <si>
     <t>ZAV02I</t>
   </si>
   <si>
-    <t>Zavicefta 2.5g Vial</t>
+    <t xml:space="preserve">Zavicefta 2.5g Vial</t>
   </si>
   <si>
     <t>CEF01I</t>
   </si>
   <si>
-    <t>Ceftriaxone 1g Vial</t>
+    <t xml:space="preserve">Ceftriaxone 1g Vial</t>
   </si>
   <si>
     <t>J01DD04</t>
   </si>
   <si>
-    <t>3rd cephas 呼吸道菌首選@ 常用量: 2 g qd@ Max: 2 g q12h</t>
+    <t xml:space="preserve">3rd cephas 呼吸道菌首選@ 常用量: 2 g qd@ Max: 2 g q12h</t>
   </si>
   <si>
     <t>ROC02I</t>
   </si>
   <si>
-    <t>Rocephin 500mg Vial#</t>
-  </si>
-  <si>
-    <t>Ceftriaxone(Rocephin) 500mg Vial#</t>
+    <t xml:space="preserve">Rocephin 500mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceftriaxone(Rocephin) 500mg Vial#</t>
   </si>
   <si>
     <t>SIN01I</t>
   </si>
   <si>
-    <t>Sintrix 500mg Vial#</t>
-  </si>
-  <si>
-    <t>Ceftriaxone(Sintrix) 500mg Vial#</t>
+    <t xml:space="preserve">Sintrix 500mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceftriaxone(Sintrix) 500mg Vial#</t>
   </si>
   <si>
     <t>CEF09O</t>
   </si>
   <si>
-    <t>Cefixmycin 100mg Cap#</t>
-  </si>
-  <si>
-    <t>Cefixime(Cefixmycin) 100mg Cap#</t>
+    <t xml:space="preserve">Cefixmycin 100mg Cap#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefixime(Cefixmycin) 100mg Cap#</t>
   </si>
   <si>
     <t>J01DD08</t>
@@ -644,67 +651,67 @@
     <t>CEX01O</t>
   </si>
   <si>
-    <t>Cexime 100mg Cap#</t>
-  </si>
-  <si>
-    <t>Cefixime(Cexime) 100mg Cap#</t>
-  </si>
-  <si>
-    <t>建議量: 400 mg qd or 200 mg q12h@ Ccr less than 50: 300 mg q12h to qd@ Ccr less than 10: 200 mg to 400 mg qd@ HD: 300 mg to 400 mg qd</t>
+    <t xml:space="preserve">Cexime 100mg Cap#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefixime(Cexime) 100mg Cap#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量: 400 mg qd or 200 mg q12h@ Ccr less than 50: 300 mg q12h to qd@ Ccr less than 10: 200 mg to 400 mg qd@ HD: 300 mg to 400 mg qd</t>
   </si>
   <si>
     <t>BRO02I</t>
   </si>
   <si>
-    <t>Brosym For Inj 2Gm/Vial</t>
-  </si>
-  <si>
-    <t>Cefoperazone+Sulbactam (Brosym) FOR INJ 2GM/VIAL</t>
+    <t xml:space="preserve">Brosym For Inj 2Gm/Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefoperazone+Sulbactam (Brosym) FOR INJ 2GM/VIAL</t>
   </si>
   <si>
     <t>J01DD62</t>
   </si>
   <si>
-    <t>無法穿透 BBB 且膽道濃度高@ 建議量: 4 g q8h@ Ccr less 30: 4 g q12h@ Ccr less 15 or HD: 2 g q12h</t>
+    <t xml:space="preserve">無法穿透 BBB 且膽道濃度高@ 建議量: 4 g q8h@ Ccr less 30: 4 g q12h@ Ccr less 15 or HD: 2 g q12h</t>
   </si>
   <si>
     <t>ANT01I</t>
   </si>
   <si>
-    <t>Antifect 1g Vial#</t>
-  </si>
-  <si>
-    <t>Cefepime (Antifect) 1000mg Vial#</t>
+    <t xml:space="preserve">Antifect 1g Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefepime (Antifect) 1000mg Vial#</t>
   </si>
   <si>
     <t>J01DE01</t>
   </si>
   <si>
-    <t>4th cephas 對ESBL失敗率高@ 建議量: 2 to 3 g q8h@ Ccr less 30: 2 g qd@ Ccr less 10 or HD: 1 g qd</t>
+    <t xml:space="preserve">4th cephas 對ESBL失敗率高@ 建議量: 2 to 3 g q8h@ Ccr less 30: 2 g qd@ Ccr less 10 or HD: 1 g qd</t>
   </si>
   <si>
     <t>MEP02I</t>
   </si>
   <si>
-    <t>Mepem 250mg Vial#</t>
-  </si>
-  <si>
-    <t>Meropenem(Mepem) 250mg Vial#</t>
+    <t xml:space="preserve">Mepem 250mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meropenem(Mepem) 250mg Vial#</t>
   </si>
   <si>
     <t>J01DH02</t>
   </si>
   <si>
-    <t>建議量: 500 mg to 1 gm q8h@ Ccr less than 50: q12h@ Ccr less than 25: 半劑量 q12h@ Ccr less than 10, HD or PD: 半劑量 qd</t>
+    <t xml:space="preserve">建議量: 500 mg to 1 gm q8h@ Ccr less than 50: q12h@ Ccr less than 25: 半劑量 q12h@ Ccr less than 10, HD or PD: 半劑量 qd</t>
   </si>
   <si>
     <t>INV01I</t>
   </si>
   <si>
-    <t>Invanz 1gm Vial#</t>
-  </si>
-  <si>
-    <t>Ertapenem(Invanz) 1gm Vial#</t>
+    <t xml:space="preserve">Invanz 1gm Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ertapenem(Invanz) 1gm Vial#</t>
   </si>
   <si>
     <t>J01DH03</t>
@@ -716,37 +723,37 @@
     <t>FIN01I</t>
   </si>
   <si>
-    <t>Finibax 0.25gm Vial#</t>
-  </si>
-  <si>
-    <t>Doripenem(Finibax) 0.25gm Vial#</t>
+    <t xml:space="preserve">Finibax 0.25gm Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doripenem(Finibax) 0.25gm Vial#</t>
   </si>
   <si>
     <t>J01DH04</t>
   </si>
   <si>
-    <t>建議量: 500 mg q8h@ P aeruginosa and  A baumannii 需要 1 gm q8h@  Ccr less than 50: 半劑量 q8h@ Ccr less than 30: 半劑量 q12h@ Ccr less than 10, HD or PD: 半劑量 qd</t>
+    <t xml:space="preserve">建議量: 500 mg q8h@ P aeruginosa and  A baumannii 需要 1 gm q8h@  Ccr less than 50: 半劑量 q8h@ Ccr less than 30: 半劑量 q12h@ Ccr less than 10, HD or PD: 半劑量 qd</t>
   </si>
   <si>
     <t>ZIN04I</t>
   </si>
   <si>
-    <t>Zinforo 600mg Vial</t>
-  </si>
-  <si>
-    <t>Ceftaroline (Zinforo) 600mg Vial</t>
+    <t xml:space="preserve">Zinforo 600mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceftaroline (Zinforo) 600mg Vial</t>
   </si>
   <si>
     <t>J01DI02</t>
   </si>
   <si>
-    <t>5th cephas 相當vanco + ceftri@ 高劑量: 600 mg q8h@ Ccr less 30: 300 mg q8h@ Ccr less 15 or HD: 200 mg q8h</t>
+    <t xml:space="preserve">5th cephas 相當vanco + ceftri@ 高劑量: 600 mg q8h@ Ccr less 30: 300 mg q8h@ Ccr less 15 or HD: 200 mg q8h</t>
   </si>
   <si>
     <t>ZER01I</t>
   </si>
   <si>
-    <t>Zerbaxa 1.5gm Vial</t>
+    <t xml:space="preserve">Zerbaxa 1.5gm Vial</t>
   </si>
   <si>
     <t>J01DI54</t>
@@ -755,25 +762,25 @@
     <t>BAK01O</t>
   </si>
   <si>
-    <t>Baktar Tab</t>
-  </si>
-  <si>
-    <t>Cotrimoxazol(Baktar) Tab</t>
+    <t xml:space="preserve">Baktar Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotrimoxazol(Baktar) Tab</t>
   </si>
   <si>
     <t>J01EE01O</t>
   </si>
   <si>
-    <t>UTI 以 fluoroquinolones 替代@ Ccr less than 30: qd@ Ccr less than 15 or HD or PD: qod</t>
+    <t xml:space="preserve">UTI 以 fluoroquinolones 替代@ Ccr less than 30: qd@ Ccr less than 15 or HD or PD: qod</t>
   </si>
   <si>
     <t>SEP02I</t>
   </si>
   <si>
-    <t>Septrin For Infusion#</t>
-  </si>
-  <si>
-    <t>Cotrimoxazol(Septrin) 5ml inj#</t>
+    <t xml:space="preserve">Septrin For Infusion#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotrimoxazol(Septrin) 5ml inj#</t>
   </si>
   <si>
     <t>J01EE01</t>
@@ -782,37 +789,37 @@
     <t>SEV01I</t>
   </si>
   <si>
-    <t>Sevatrim 5ml Amp#</t>
-  </si>
-  <si>
-    <t>Cotrimoxazol(Sevatrim) 5ml Amp#</t>
-  </si>
-  <si>
-    <t>iv drip over than 1hr@ 5 mg TMP per kg q6 to 8h@ Ccr less than 30: qd@ Ccr less than 15 or HD or PD: qod</t>
+    <t xml:space="preserve">Sevatrim 5ml Amp#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotrimoxazol(Sevatrim) 5ml Amp#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iv drip over than 1hr@ 5 mg TMP per kg q6 to 8h@ Ccr less than 30: qd@ Ccr less than 15 or HD or PD: qod</t>
   </si>
   <si>
     <t>SUL01S</t>
   </si>
   <si>
-    <t>Sulfacotrim Susp 60ml Bot#</t>
-  </si>
-  <si>
-    <t>Cotrimoxazol(Sulfacotrim) Susp 60ml Bot#</t>
+    <t xml:space="preserve">Sulfacotrim Susp 60ml Bot#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotrimoxazol(Sulfacotrim) Susp 60ml Bot#</t>
   </si>
   <si>
     <t>J01EE01S</t>
   </si>
   <si>
-    <t>4 mg TMP per kg q12h@ 預防 UTI: 2 mg TMP per kg qd</t>
+    <t xml:space="preserve">4 mg TMP per kg q12h@ 預防 UTI: 2 mg TMP per kg qd</t>
   </si>
   <si>
     <t>ERO01O</t>
   </si>
   <si>
-    <t>Erythromycin 250mg Tab#(舊)</t>
-  </si>
-  <si>
-    <t>Erythromycin 250mg Tab#</t>
+    <t xml:space="preserve">Erythromycin 250mg Tab#(舊)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erythromycin 250mg Tab#</t>
   </si>
   <si>
     <t>J01FA01</t>
@@ -821,7 +828,7 @@
     <t>ERY03O</t>
   </si>
   <si>
-    <t>Erythromycin 250mg Cap#</t>
+    <t xml:space="preserve">Erythromycin 250mg Cap#</t>
   </si>
   <si>
     <t xml:space="preserve">建議量: 500 mg q6h@ 小兒; 10 mg per kg q6h@ 抑制 statins 代謝及 theophylline 排除@ 留意 DDI 誘發 TdP </t>
@@ -830,112 +837,112 @@
     <t>CLA04O</t>
   </si>
   <si>
-    <t>Claricin 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Clarithromycin (Claricin) 250mg Tab#</t>
+    <t xml:space="preserve">Claricin 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarithromycin (Claricin) 250mg Tab#</t>
   </si>
   <si>
     <t>J01FA09</t>
   </si>
   <si>
-    <t>建議量: 500 mg q12h@ Ccr less than 30: 500 mg qd@ Ccr less than 10, HD or PD: 250 mg qd</t>
+    <t xml:space="preserve">建議量: 500 mg q12h@ Ccr less than 30: 500 mg qd@ Ccr less than 10, HD or PD: 250 mg qd</t>
   </si>
   <si>
     <t>KLA01O</t>
   </si>
   <si>
-    <t>Klaricid XL 500mg Tab#</t>
-  </si>
-  <si>
-    <t>Clarithromycin(Klaricid XL) 500mg Tab#</t>
+    <t xml:space="preserve">Klaricid XL 500mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarithromycin(Klaricid XL) 500mg Tab#</t>
   </si>
   <si>
     <t>J01FA09R</t>
   </si>
   <si>
-    <t>建議量: 1 gm qd@ 須飯後</t>
+    <t xml:space="preserve">建議量: 1 gm qd@ 須飯後</t>
   </si>
   <si>
     <t>KLA02O</t>
   </si>
   <si>
-    <t>Klaricid 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Clarithromycin(Klaricid) 250mg Tab#</t>
+    <t xml:space="preserve">Klaricid 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarithromycin(Klaricid) 250mg Tab#</t>
   </si>
   <si>
     <t>KLA03O</t>
   </si>
   <si>
-    <t>Klarith F.C. 250MG Tab#</t>
-  </si>
-  <si>
-    <t>Clarithromycin (Klarith) 250mg Tab#</t>
+    <t xml:space="preserve">Klarith F.C. 250MG Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarithromycin (Klarith) 250mg Tab#</t>
   </si>
   <si>
     <t>ULI01O</t>
   </si>
   <si>
-    <t>Ulicin 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Clarithromycin(Ulicin) 250mg Tab</t>
+    <t xml:space="preserve">Ulicin 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarithromycin(Ulicin) 250mg Tab</t>
   </si>
   <si>
     <t>AZI01S</t>
   </si>
   <si>
-    <t>Azithrom Susp 40mg/mL;15mL</t>
-  </si>
-  <si>
-    <t>Azithromycin (Azithrom) Susp 40mg/ml 15ml#</t>
+    <t xml:space="preserve">Azithrom Susp 40mg/mL;15mL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azithromycin (Azithrom) Susp 40mg/ml 15ml#</t>
   </si>
   <si>
     <t>J01FA10S</t>
   </si>
   <si>
-    <t>須空腹@ 10 mg per kg qd for 3 days@ loading: 10 mg per kg then 5 mg per kg for 4 days</t>
+    <t xml:space="preserve">須空腹@ 10 mg per kg qd for 3 days@ loading: 10 mg per kg then 5 mg per kg for 4 days</t>
   </si>
   <si>
     <t>AZI02O</t>
   </si>
   <si>
-    <t>Aziciin 250mg Tab</t>
-  </si>
-  <si>
-    <t>Azithromycin(Aziciin) 250mg Tab</t>
+    <t xml:space="preserve">Aziciin 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azithromycin(Aziciin) 250mg Tab</t>
   </si>
   <si>
     <t>J01FA10</t>
   </si>
   <si>
-    <t>500 mg qd for 3 days@ Legionnaires disease for 1 week</t>
+    <t xml:space="preserve">500 mg qd for 3 days@ Legionnaires disease for 1 week</t>
   </si>
   <si>
     <t>ZIT01O</t>
   </si>
   <si>
-    <t>Zithromax 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Azithromycin(Zithromax) 250mg Tab#</t>
+    <t xml:space="preserve">Zithromax 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azithromycin(Zithromax) 250mg Tab#</t>
   </si>
   <si>
     <t>ZIT01S</t>
   </si>
   <si>
-    <t>Zithromax Susp 40mg/ml;15ml#</t>
-  </si>
-  <si>
-    <t>Azithromycin(Zithromax) Susp 40mg/ml 15ml#</t>
+    <t xml:space="preserve">Zithromax Susp 40mg/ml;15ml#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azithromycin(Zithromax) Susp 40mg/ml 15ml#</t>
   </si>
   <si>
     <t>CLI01I</t>
   </si>
   <si>
-    <t>Clindamycin 300mg/2ml Amp</t>
+    <t xml:space="preserve">Clindamycin 300mg/2ml Amp</t>
   </si>
   <si>
     <t>J01FF01</t>
@@ -944,166 +951,166 @@
     <t>CLI02I</t>
   </si>
   <si>
-    <t>Clincin Inj. 300mg/2ml Amp</t>
-  </si>
-  <si>
-    <t>Clindamycin(Clincin) 300mg/2ml Amp</t>
-  </si>
-  <si>
-    <t>建議量: 900 mg to 600 mg q8h@ 小兒: 13 mg per kg q8h@ 10% 經 urine 排除</t>
+    <t xml:space="preserve">Clincin Inj. 300mg/2ml Amp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clindamycin(Clincin) 300mg/2ml Amp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量: 900 mg to 600 mg q8h@ 小兒: 13 mg per kg q8h@ 10% 經 urine 排除</t>
   </si>
   <si>
     <t>LIN03O</t>
   </si>
   <si>
-    <t>Lindacin 150mg Cap</t>
-  </si>
-  <si>
-    <t>Clindamycin(Lindacin) 150mg Cap</t>
+    <t xml:space="preserve">Lindacin 150mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clindamycin(Lindacin) 150mg Cap</t>
   </si>
   <si>
     <t>J01FF01O</t>
   </si>
   <si>
-    <t>建議量: 450 mg q6h@ 小兒: 10 mg per kg q8h</t>
+    <t xml:space="preserve">建議量: 450 mg q6h@ 小兒: 10 mg per kg q8h</t>
   </si>
   <si>
     <t>VGE01I</t>
   </si>
   <si>
-    <t>V-Genta 80mg/2ml Vial</t>
-  </si>
-  <si>
-    <t>Gentamicin(V-Genta) 80mg/2ml Vial</t>
+    <t xml:space="preserve">V-Genta 80mg/2ml Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gentamicin(V-Genta) 80mg/2ml Vial</t>
   </si>
   <si>
     <t>J01GB03</t>
   </si>
   <si>
-    <t>建議量: 1.7 mg per kg q8h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
+    <t xml:space="preserve">建議量: 1.7 mg per kg q8h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
   </si>
   <si>
     <t>NEO02O</t>
   </si>
   <si>
-    <t>Neomycin 250mg Cap</t>
+    <t xml:space="preserve">Neomycin 250mg Cap</t>
   </si>
   <si>
     <t>J01GB05</t>
   </si>
   <si>
-    <t>500 mg bid@ abs: poor</t>
+    <t xml:space="preserve">500 mg bid@ abs: poor</t>
   </si>
   <si>
     <t>ACE01I</t>
   </si>
   <si>
-    <t>Acemycin 500mg/2ml Vial#</t>
-  </si>
-  <si>
-    <t>Amikacin(Acemycin) 500mg/2ml Vial#</t>
+    <t xml:space="preserve">Acemycin 500mg/2ml Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amikacin(Acemycin) 500mg/2ml Vial#</t>
   </si>
   <si>
     <t>J01GB06</t>
   </si>
   <si>
-    <t>建議量: 7.5 mg per kg q12h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
+    <t xml:space="preserve">建議量: 7.5 mg per kg q12h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
   </si>
   <si>
     <t>CIN01I</t>
   </si>
   <si>
-    <t>Cinolone 200mg/100ml Vial</t>
-  </si>
-  <si>
-    <t>Ciprofloxacin(Cinolone) 200mg/100ml Bot</t>
+    <t xml:space="preserve">Cinolone 200mg/100ml Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciprofloxacin(Cinolone) 200mg/100ml Bot</t>
   </si>
   <si>
     <t>J01MA02</t>
   </si>
   <si>
-    <t>建議量: 400 mg q12h@ Ccr less than 30, HD or PD: qd</t>
+    <t xml:space="preserve">建議量: 400 mg q12h@ Ccr less than 30, HD or PD: qd</t>
   </si>
   <si>
     <t>CIN02O</t>
   </si>
   <si>
-    <t>Cinolone 250mg Tab</t>
-  </si>
-  <si>
-    <t>Ciprofloxacin(Cinolone) 250mg Tab#</t>
+    <t xml:space="preserve">Cinolone 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciprofloxacin(Cinolone) 250mg Tab#</t>
   </si>
   <si>
     <t>J01MA02O</t>
   </si>
   <si>
-    <t>建議量: 500 mg q12h 須空腹@ Ccr less than 30, HD or PD: qd</t>
+    <t xml:space="preserve">建議量: 500 mg q12h 須空腹@ Ccr less than 30, HD or PD: qd</t>
   </si>
   <si>
     <t>CIP01O</t>
   </si>
   <si>
-    <t>Ciproxin 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Ciprofloxacin(Ciproxin) 250mg Tab#</t>
+    <t xml:space="preserve">Ciproxin 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciprofloxacin(Ciproxin) 250mg Tab#</t>
   </si>
   <si>
     <t>CIP02I</t>
   </si>
   <si>
-    <t>Ciproxin 200MG/100ML BOT</t>
-  </si>
-  <si>
-    <t>Ciprofloxacin(Ciproxin) 200mg/100ml Bot#</t>
+    <t xml:space="preserve">Ciproxin 200MG/100ML BOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciprofloxacin(Ciproxin) 200mg/100ml Bot#</t>
   </si>
   <si>
     <t>CRA02O</t>
   </si>
   <si>
-    <t>Cravit 500mg Tab#</t>
-  </si>
-  <si>
-    <t>Levofloxacin(Cravit) 500mg Tab#</t>
+    <t xml:space="preserve">Cravit 500mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levofloxacin(Cravit) 500mg Tab#</t>
   </si>
   <si>
     <t>J01MA12O</t>
   </si>
   <si>
-    <t>建議量: 500 mg qd@  Ccr less than 50: 半劑量 qd@ Ccr less than 20, HD or PD: 半劑量 qod</t>
+    <t xml:space="preserve">建議量: 500 mg qd@  Ccr less than 50: 半劑量 qd@ Ccr less than 20, HD or PD: 半劑量 qod</t>
   </si>
   <si>
     <t>CRA03I</t>
   </si>
   <si>
-    <t>Cravit 500mg/100ml Vial#</t>
-  </si>
-  <si>
-    <t>Levofloxacin(Cravit) 500mg/100ml Vial#</t>
+    <t xml:space="preserve">Cravit 500mg/100ml Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levofloxacin(Cravit) 500mg/100ml Vial#</t>
   </si>
   <si>
     <t>J01MA12</t>
   </si>
   <si>
-    <t>建議量: 500 mg to 750 mg qd@ Ccr less than 50: 半劑量 qd@ Ccr less than 20, HD or PD: 半劑量 qod</t>
+    <t xml:space="preserve">建議量: 500 mg to 750 mg qd@ Ccr less than 50: 半劑量 qd@ Ccr less than 20, HD or PD: 半劑量 qod</t>
   </si>
   <si>
     <t>LEV03O</t>
   </si>
   <si>
-    <t>Levonolon 500mg Tab(公費)</t>
-  </si>
-  <si>
-    <t>Levofloxacin(Levonolon) 500mg Tab(公費)</t>
+    <t xml:space="preserve">Levonolon 500mg Tab(公費)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levofloxacin(Levonolon) 500mg Tab(公費)</t>
   </si>
   <si>
     <t>AVE01I</t>
   </si>
   <si>
-    <t>Avelox 400mg/250ml#</t>
-  </si>
-  <si>
-    <t>Moxifloxacin(Avelox) 400mg/250ml#</t>
+    <t xml:space="preserve">Avelox 400mg/250ml#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moxifloxacin(Avelox) 400mg/250ml#</t>
   </si>
   <si>
     <t>J01MA14</t>
@@ -1115,10 +1122,10 @@
     <t>AVE01O</t>
   </si>
   <si>
-    <t>Avelox 400mg Tab#</t>
-  </si>
-  <si>
-    <t>Moxifloxacin(Avelox) 400mg Tab#</t>
+    <t xml:space="preserve">Avelox 400mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moxifloxacin(Avelox) 400mg Tab#</t>
   </si>
   <si>
     <t>J01MA14O</t>
@@ -1127,73 +1134,73 @@
     <t>FLO02O</t>
   </si>
   <si>
-    <t>Floxsafe 400mg Tab (公費)</t>
-  </si>
-  <si>
-    <t>Moxifloxacin(Floxsafe) 400mg Tab (公費)</t>
+    <t xml:space="preserve">Floxsafe 400mg Tab (公費)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moxifloxacin(Floxsafe) 400mg Tab (公費)</t>
   </si>
   <si>
     <t>MOS01I</t>
   </si>
   <si>
-    <t>Mosflow 400mg/250ml Bot</t>
-  </si>
-  <si>
-    <t>Moxifloxacin(Mosflow) 400mg/250ml Bot</t>
+    <t xml:space="preserve">Mosflow 400mg/250ml Bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moxifloxacin(Mosflow) 400mg/250ml Bot</t>
   </si>
   <si>
     <t>MOS01O</t>
   </si>
   <si>
-    <t>Mosflow 400mg Tab</t>
-  </si>
-  <si>
-    <t>Moxifloxacin(Mosflow) 400mg Tab#</t>
+    <t xml:space="preserve">Mosflow 400mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moxifloxacin(Mosflow) 400mg Tab#</t>
   </si>
   <si>
     <t>DOL02O</t>
   </si>
   <si>
-    <t>Dolcol 250mg Tab</t>
-  </si>
-  <si>
-    <t>Pipemidic Acid(Dolcol) 250mg Tab</t>
+    <t xml:space="preserve">Dolcol 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pipemidic Acid(Dolcol) 250mg Tab</t>
   </si>
   <si>
     <t>J01MB04</t>
   </si>
   <si>
-    <t>仿單: 500 mg to 2 gm daily dosage</t>
+    <t xml:space="preserve">仿單: 500 mg to 2 gm daily dosage</t>
   </si>
   <si>
     <t>TAI01O</t>
   </si>
   <si>
-    <t>Taigexyn 250mg Cap</t>
-  </si>
-  <si>
-    <t>Nemonoxacin (Taigexyn) 250mg Cap</t>
+    <t xml:space="preserve">Taigexyn 250mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nemonoxacin (Taigexyn) 250mg Cap</t>
   </si>
   <si>
     <t>J01MB08</t>
   </si>
   <si>
-    <t>仿單: 500 mg once  daily@ SE: 肌腱炎、肌腱斷裂、周邊神經炎@ DDI: TdP</t>
+    <t xml:space="preserve">仿單: 500 mg once  daily@ SE: 肌腱炎、肌腱斷裂、周邊神經炎@ DDI: TdP</t>
   </si>
   <si>
     <t>TAI06I</t>
   </si>
   <si>
-    <t>Taigexyn 500mg/250ml Bag</t>
-  </si>
-  <si>
-    <t>Nemonoxacin (Taigexyn) 500mg/250ml Bag</t>
+    <t xml:space="preserve">Taigexyn 500mg/250ml Bag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nemonoxacin (Taigexyn) 500mg/250ml Bag</t>
   </si>
   <si>
     <t>VAN03I</t>
   </si>
   <si>
-    <t>Vancomycin 1g Vial#</t>
+    <t xml:space="preserve">Vancomycin 1g Vial#</t>
   </si>
   <si>
     <t>J01XA01</t>
@@ -1202,37 +1209,37 @@
     <t>VAN04I</t>
   </si>
   <si>
-    <t>Vanco 1g Vial</t>
-  </si>
-  <si>
-    <t>Vancomycin(Vanco) 1g Vial</t>
-  </si>
-  <si>
-    <t>建議量: 1 gm or 15 mg per kg q12h@ 使用超過二周須監測血中濃度</t>
+    <t xml:space="preserve">Vanco 1g Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vancomycin(Vanco) 1g Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量: 1 gm or 15 mg per kg q12h@ 使用超過二周須監測血中濃度</t>
   </si>
   <si>
     <t>VAN04O</t>
   </si>
   <si>
-    <t>Vancover 125mg Cap</t>
-  </si>
-  <si>
-    <t>Vancomyin(Vancover) 125mg Cap</t>
+    <t xml:space="preserve">Vancover 125mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vancomyin(Vancover) 125mg Cap</t>
   </si>
   <si>
     <t>J01XA01O</t>
   </si>
   <si>
-    <t>建議量: 125 mg or 500 mg q6h for 10 days</t>
+    <t xml:space="preserve">建議量: 125 mg or 500 mg q6h for 10 days</t>
   </si>
   <si>
     <t>TAR02I</t>
   </si>
   <si>
-    <t>Targocid 200mg Vial#</t>
-  </si>
-  <si>
-    <t>Teicoplanin(Targocid) 200mg Vial#</t>
+    <t xml:space="preserve">Targocid 200mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teicoplanin(Targocid) 200mg Vial#</t>
   </si>
   <si>
     <t>J01XA02</t>
@@ -1244,19 +1251,19 @@
     <t>TEI01I</t>
   </si>
   <si>
-    <t>Teicod 200mg Vial</t>
-  </si>
-  <si>
-    <t>Teicoplanin(Teicod) 200mg Vial</t>
+    <t xml:space="preserve">Teicod 200mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teicoplanin(Teicod) 200mg Vial</t>
   </si>
   <si>
     <t>COL02I</t>
   </si>
   <si>
-    <t>Colimycin 2MU Vial</t>
-  </si>
-  <si>
-    <t>Colistin(Colimycin) 2MU Vial</t>
+    <t xml:space="preserve">Colimycin 2MU Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colistin(Colimycin) 2MU Vial</t>
   </si>
   <si>
     <t>J01XB01</t>
@@ -1268,34 +1275,34 @@
     <t>FUC01O</t>
   </si>
   <si>
-    <t>Fucidin 250mg Tab#</t>
-  </si>
-  <si>
-    <t>Fusidate(Fucidin) 250mg Tab#</t>
+    <t xml:space="preserve">Fucidin 250mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusidate(Fucidin) 250mg Tab#</t>
   </si>
   <si>
     <t>J01XC01</t>
   </si>
   <si>
-    <t>建議量: 500 mg q12h@ 小兒: 10 mg per kg q12h</t>
+    <t xml:space="preserve">建議量: 500 mg q12h@ 小兒: 10 mg per kg q12h</t>
   </si>
   <si>
     <t>FUS01O</t>
   </si>
   <si>
-    <t>Fusodate 250mg Tab</t>
-  </si>
-  <si>
-    <t>Fusidate(Fusodate) 250mg Tab</t>
+    <t xml:space="preserve">Fusodate 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusidate(Fusodate) 250mg Tab</t>
   </si>
   <si>
     <t>DYN02O</t>
   </si>
   <si>
-    <t>Dynin 250mg Tab</t>
-  </si>
-  <si>
-    <t>Metronidazole(Dynin) 250mg Tab</t>
+    <t xml:space="preserve">Dynin 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metronidazole(Dynin) 250mg Tab</t>
   </si>
   <si>
     <t>J01XD01</t>
@@ -1304,337 +1311,337 @@
     <t>FLA01O</t>
   </si>
   <si>
-    <t>Flagyl 250mg Tab</t>
-  </si>
-  <si>
-    <t>Metronidazole(Flagyl) 250mg Tab</t>
+    <t xml:space="preserve">Flagyl 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metronidazole(Flagyl) 250mg Tab</t>
   </si>
   <si>
     <t>MET06I</t>
   </si>
   <si>
-    <t>Metronidazole 500mg/100ml</t>
-  </si>
-  <si>
-    <t>Max: 4 gm per day@ Ccr less than 10, HD or Child C: 50%</t>
+    <t xml:space="preserve">Metronidazole 500mg/100ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max: 4 gm per day@ Ccr less than 10, HD or Child C: 50%</t>
   </si>
   <si>
     <t>MET18O</t>
   </si>
   <si>
-    <t>Metrozole 250mg Tab</t>
-  </si>
-  <si>
-    <t>Metronidazole(Metrozole) 250mg Tab</t>
+    <t xml:space="preserve">Metrozole 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metronidazole(Metrozole) 250mg Tab</t>
   </si>
   <si>
     <t>SAB01I</t>
   </si>
   <si>
-    <t>SABS 500mg/100ml Bot</t>
-  </si>
-  <si>
-    <t>Metronidazole(SABS) 500mg/100ml Bot</t>
+    <t xml:space="preserve">SABS 500mg/100ml Bot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metronidazole(SABS) 500mg/100ml Bot</t>
   </si>
   <si>
     <t>FOL01I</t>
   </si>
   <si>
-    <t>Folsmycin powder for injection#</t>
-  </si>
-  <si>
-    <t>Fosfomycin powder for injection (Folsmycin)</t>
+    <t xml:space="preserve">Folsmycin powder for injection#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fosfomycin powder for injection (Folsmycin)</t>
   </si>
   <si>
     <t>J01XX01</t>
   </si>
   <si>
-    <t>仿單: 2 to 4 gm daily dosage@ 小兒: 100 to 200 mg per kg daily dosage@ Ccr less than 30: 60%</t>
+    <t xml:space="preserve">仿單: 2 to 4 gm daily dosage@ 小兒: 100 to 200 mg per kg daily dosage@ Ccr less than 30: 60%</t>
   </si>
   <si>
     <t>MON04O</t>
   </si>
   <si>
-    <t>Monurol Granular Powder#</t>
-  </si>
-  <si>
-    <t>Fosfomycin(Monurol) Granular Powder#</t>
+    <t xml:space="preserve">Monurol Granular Powder#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fosfomycin(Monurol) Granular Powder#</t>
   </si>
   <si>
     <t>LIN04O</t>
   </si>
   <si>
-    <t>Linetero 600mg Tab</t>
-  </si>
-  <si>
-    <t>Linezolid(Linetero) 600mg Tab#</t>
+    <t xml:space="preserve">Linetero 600mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linezolid(Linetero) 600mg Tab#</t>
   </si>
   <si>
     <t>J01XX08O</t>
   </si>
   <si>
-    <t>建議量: 600 mg q12h 須空腹</t>
+    <t xml:space="preserve">建議量: 600 mg q12h 須空腹</t>
   </si>
   <si>
     <t>ZYV01I</t>
   </si>
   <si>
-    <t>Zyvox 600mg/300ml Bag#</t>
-  </si>
-  <si>
-    <t>Linezolid(Zyvox) 600mg/300ml Bag#</t>
+    <t xml:space="preserve">Zyvox 600mg/300ml Bag#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linezolid(Zyvox) 600mg/300ml Bag#</t>
   </si>
   <si>
     <t>J01XX08</t>
   </si>
   <si>
-    <t>建議量: 600 mg q12h</t>
+    <t xml:space="preserve">建議量: 600 mg q12h</t>
   </si>
   <si>
     <t>ZYV01O</t>
   </si>
   <si>
-    <t>Zyvox 600mg Tab#</t>
-  </si>
-  <si>
-    <t>Linezolid(Zyvox) 600mg Tab#</t>
+    <t xml:space="preserve">Zyvox 600mg Tab#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linezolid(Zyvox) 600mg Tab#</t>
   </si>
   <si>
     <t>CUB01I</t>
   </si>
   <si>
-    <t>Cubicin 500mg Vial</t>
-  </si>
-  <si>
-    <t>Daptomycin(Cubicin) 500mg Vial</t>
+    <t xml:space="preserve">Cubicin 500mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daptomycin(Cubicin) 500mg Vial</t>
   </si>
   <si>
     <t>J01XX09</t>
   </si>
   <si>
-    <t>組織穿透差不適 pneumonia@ endocarditis: 8 to 12 mg per kg qd@ soft tissue: 4 to 6 mg per kg qd@ Ccr less than 30, HD or PD: qod@ DDI: statins following up CPK</t>
+    <t xml:space="preserve">組織穿透差不適 pneumonia@ endocarditis: 8 to 12 mg per kg qd@ soft tissue: 4 to 6 mg per kg qd@ Ccr less than 30, HD or PD: qod@ DDI: statins following up CPK</t>
   </si>
   <si>
     <t>AMB01I</t>
   </si>
   <si>
-    <t>Ambisome 50mg Vial#</t>
-  </si>
-  <si>
-    <t>Amphotericin B Liposome(Ambisome) 50mg Vial#</t>
+    <t xml:space="preserve">Ambisome 50mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amphotericin B Liposome(Ambisome) 50mg Vial#</t>
   </si>
   <si>
     <t>J02AA01</t>
   </si>
   <si>
-    <t>建議量: 3 to 6 mg per kg once daily</t>
+    <t xml:space="preserve">建議量: 3 to 6 mg per kg once daily</t>
   </si>
   <si>
     <t>AMP02I</t>
   </si>
   <si>
-    <t>Ampholipad 50mg Vial</t>
-  </si>
-  <si>
-    <t>Amphotericin B Liposome(Ampholipad) 50mg Vial</t>
+    <t xml:space="preserve">Ampholipad 50mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amphotericin B Liposome(Ampholipad) 50mg Vial</t>
   </si>
   <si>
     <t>FUN01I</t>
   </si>
   <si>
-    <t>Fungizone 50mg Vial</t>
-  </si>
-  <si>
-    <t>AmphotericinB(Fungizone) 50mg Vial</t>
-  </si>
-  <si>
-    <t>建議量: 0.5 to 1.5 mg per kg once daily</t>
+    <t xml:space="preserve">Fungizone 50mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AmphotericinB(Fungizone) 50mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">建議量: 0.5 to 1.5 mg per kg once daily</t>
   </si>
   <si>
     <t>DIF01I</t>
   </si>
   <si>
-    <t>Diflucan 100mg/50ml Vial#</t>
-  </si>
-  <si>
-    <t>Fluconazole(Diflucan) 100mg/50ml Vial#</t>
+    <t xml:space="preserve">Diflucan 100mg/50ml Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluconazole(Diflucan) 100mg/50ml Vial#</t>
   </si>
   <si>
     <t>J02AC01</t>
   </si>
   <si>
-    <t>建議量: 200 to 800 mg daily@ Ccr less than 50: 劑量減半@ Ccr less 25: 四分之一劑量@ HD:  洗完正常量</t>
+    <t xml:space="preserve">建議量: 200 to 800 mg daily@ Ccr less than 50: 劑量減半@ Ccr less 25: 四分之一劑量@ HD:  洗完正常量</t>
   </si>
   <si>
     <t>FLU06O</t>
   </si>
   <si>
-    <t>Fluene 50mg Cap#</t>
-  </si>
-  <si>
-    <t>Fluconazole(Fluene) 50mg Cap#</t>
+    <t xml:space="preserve">Fluene 50mg Cap#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluconazole(Fluene) 50mg Cap#</t>
   </si>
   <si>
     <t>FLU11O</t>
   </si>
   <si>
-    <t>Flucozyd 200mg Cap</t>
-  </si>
-  <si>
-    <t>Fluconazole(Flucozyd) 200mg Cap</t>
+    <t xml:space="preserve">Flucozyd 200mg Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluconazole(Flucozyd) 200mg Cap</t>
   </si>
   <si>
     <t>SPO01O</t>
   </si>
   <si>
-    <t>Sporanox 100mg Cap#</t>
-  </si>
-  <si>
-    <t>Itraconazole(Sporanox) 100mg Cap#</t>
+    <t xml:space="preserve">Sporanox 100mg Cap#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Itraconazole(Sporanox) 100mg Cap#</t>
   </si>
   <si>
     <t>J02AC02</t>
   </si>
   <si>
-    <t>建議量: 200 mg qd to q12h@ DDI: QTc prolongation@ 禁忌: HF</t>
+    <t xml:space="preserve">建議量: 200 mg qd to q12h@ DDI: QTc prolongation@ 禁忌: HF</t>
   </si>
   <si>
     <t>VFE01I</t>
   </si>
   <si>
-    <t>Vfend 200mg Vial</t>
-  </si>
-  <si>
-    <t>Voriconazole (Vfend) 200mg Vial</t>
+    <t xml:space="preserve">Vfend 200mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voriconazole (Vfend) 200mg Vial</t>
   </si>
   <si>
     <t>J02AC03</t>
   </si>
   <si>
-    <t>for Aspergilllosis@ 可穿透BBB@ loading: 6 mg per kg for 2 doses than 4 mg per kg q12h@ PK: urine less than 2%@ DDI: QTc prolongation</t>
+    <t xml:space="preserve">for Aspergilllosis@ 可穿透BBB@ loading: 6 mg per kg for 2 doses than 4 mg per kg q12h@ PK: urine less than 2%@ DDI: QTc prolongation</t>
   </si>
   <si>
     <t>VFE01O</t>
   </si>
   <si>
-    <t>Vfend 200mg Tab</t>
-  </si>
-  <si>
-    <t>Voriconazole(Vfend) 200mg Tab</t>
+    <t xml:space="preserve">Vfend 200mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voriconazole(Vfend) 200mg Tab</t>
   </si>
   <si>
     <t>J02AC03O</t>
   </si>
   <si>
-    <t>須空腹因高脂食物@ 體重超過40公斤: loading: 400 mg for 2 doses than 200 mg q12h@ wt less than 40 kg: 劑量減半@ DDI: QTc prolongation</t>
+    <t xml:space="preserve">須空腹因高脂食物@ 體重超過40公斤: loading: 400 mg for 2 doses than 200 mg q12h@ wt less than 40 kg: 劑量減半@ DDI: QTc prolongation</t>
   </si>
   <si>
     <t>POS04O</t>
   </si>
   <si>
-    <t>Posanol 100mg Tab</t>
-  </si>
-  <si>
-    <t>Posaconazole(Posanol) 100mg Tab</t>
+    <t xml:space="preserve">Posanol 100mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posaconazole(Posanol) 100mg Tab</t>
   </si>
   <si>
     <t>J02AC04</t>
   </si>
   <si>
-    <t>須餐後因高脂食物增加吸收@ 建議量: 400 mg q12h@ DDI: TdP</t>
+    <t xml:space="preserve">須餐後因高脂食物增加吸收@ 建議量: 400 mg q12h@ DDI: TdP</t>
   </si>
   <si>
     <t>FLU02O</t>
   </si>
   <si>
-    <t>Flusine 500mg Tab</t>
-  </si>
-  <si>
-    <t>Flucytosine (Flusine)500mg Tab</t>
+    <t xml:space="preserve">Flusine 500mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flucytosine (Flusine)500mg Tab</t>
   </si>
   <si>
     <t>J02AX01</t>
   </si>
   <si>
-    <t>建議量: 25 mg per kg q6h@ Ccr less than 40: q12h@ Ccr less than 20: qd@ Ccr less than 10, HD or PD: qod@ 罕單用經肝臟排泄@ SE: 骨髓抑制@ 禁忌: 孕婦</t>
+    <t xml:space="preserve">建議量: 25 mg per kg q6h@ Ccr less than 40: q12h@ Ccr less than 20: qd@ Ccr less than 10, HD or PD: qod@ 罕單用經肝臟排泄@ SE: 骨髓抑制@ 禁忌: 孕婦</t>
   </si>
   <si>
     <t>MYC01I</t>
   </si>
   <si>
-    <t>Mycamine 50mg Vial#</t>
-  </si>
-  <si>
-    <t>Micafungin(Mycamine) 50mg Vial#</t>
+    <t xml:space="preserve">Mycamine 50mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micafungin(Mycamine) 50mg Vial#</t>
   </si>
   <si>
     <t>J02AX05</t>
   </si>
   <si>
-    <t>建議量: 100 mg to 150 mg qd@ 小兒: 2 to 3 mg per kg qd</t>
+    <t xml:space="preserve">建議量: 100 mg to 150 mg qd@ 小兒: 2 to 3 mg per kg qd</t>
   </si>
   <si>
     <t>ERA01I</t>
   </si>
   <si>
-    <t>Eraxis 100mg Vial#</t>
-  </si>
-  <si>
-    <t>Anidulafungin (Eraxis) 100mg Vial#</t>
+    <t xml:space="preserve">Eraxis 100mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anidulafungin (Eraxis) 100mg Vial#</t>
   </si>
   <si>
     <t>J02AX06</t>
   </si>
   <si>
-    <t>loading: 100 to 200 mg than 50 to 100 mg qd@ flow rate: less 1.1 mg per min 因副作用@ DDI: QTc prolongation</t>
+    <t xml:space="preserve">loading: 100 to 200 mg than 50 to 100 mg qd@ flow rate: less 1.1 mg per min 因副作用@ DDI: QTc prolongation</t>
   </si>
   <si>
     <t>ACY02O</t>
   </si>
   <si>
-    <t>Acylo 400mg Tab</t>
-  </si>
-  <si>
-    <t>Acyclovir(Acylo) 400mg Tab</t>
+    <t xml:space="preserve">Acylo 400mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acyclovir(Acylo) 400mg Tab</t>
   </si>
   <si>
     <t>J05AB01O</t>
   </si>
   <si>
-    <t>abs. 15% to 30%@ 建議量: 800 mg q4h@ Ccr less than 25: 800 mg q8h@ Ccr less than 10, HD or PD: 800 mg q12h</t>
+    <t xml:space="preserve">abs. 15% to 30%@ 建議量: 800 mg q4h@ Ccr less than 25: 800 mg q8h@ Ccr less than 10, HD or PD: 800 mg q12h</t>
   </si>
   <si>
     <t>ASI02I</t>
   </si>
   <si>
-    <t>Asimplex 250mg Vial</t>
-  </si>
-  <si>
-    <t>Acyclovir (Asimplex) 250mg Vial</t>
+    <t xml:space="preserve">Asimplex 250mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acyclovir (Asimplex) 250mg Vial</t>
   </si>
   <si>
     <t>J05AB01</t>
   </si>
   <si>
-    <t>建議量: 10 mg per kg q8h@ 小兒: 20 mg per kg q8h@ Ccr less than 50: q12h@ Ccr less than 25: qd@ Ccr less than 10, HD or PD: 劑量減半 qd</t>
+    <t xml:space="preserve">建議量: 10 mg per kg q8h@ 小兒: 20 mg per kg q8h@ Ccr less than 50: q12h@ Ccr less than 25: qd@ Ccr less than 10, HD or PD: 劑量減半 qd</t>
   </si>
   <si>
     <t>ZOV01I</t>
   </si>
   <si>
-    <t>Zovirax 250mg Vial</t>
-  </si>
-  <si>
-    <t>Acyclovir(Zovirax) 250mg Vial</t>
+    <t xml:space="preserve">Zovirax 250mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acyclovir(Zovirax) 250mg Vial</t>
   </si>
   <si>
     <t>CYM01I</t>
   </si>
   <si>
-    <t>Cymevene 500mg Vial#</t>
-  </si>
-  <si>
-    <t>Ganciclovir(Cymevene) 500mg Vial#</t>
+    <t xml:space="preserve">Cymevene 500mg Vial#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ganciclovir(Cymevene) 500mg Vial#</t>
   </si>
   <si>
     <t>J05AB06</t>
@@ -1643,19 +1650,19 @@
     <t>GAN01I</t>
   </si>
   <si>
-    <t>Gancicure Lyo 500mg Vial</t>
-  </si>
-  <si>
-    <t>Ganciclovir(Gancicure Lyo) 500mg Vial</t>
+    <t xml:space="preserve">Gancicure Lyo 500mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ganciclovir(Gancicure Lyo) 500mg Vial</t>
   </si>
   <si>
     <t>FAM02O</t>
   </si>
   <si>
-    <t>Famvir 250mg Tab</t>
-  </si>
-  <si>
-    <t>Famciclovir(Famvir) 250mg Tab</t>
+    <t xml:space="preserve">Famvir 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Famciclovir(Famvir) 250mg Tab</t>
   </si>
   <si>
     <t>J05AB09</t>
@@ -1664,10 +1671,10 @@
     <t>VAL05O</t>
   </si>
   <si>
-    <t>Valtrex 500mg Tab</t>
-  </si>
-  <si>
-    <t>Valaciclovir(Valtrex) 500mg Tab</t>
+    <t xml:space="preserve">Valtrex 500mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valaciclovir(Valtrex) 500mg Tab</t>
   </si>
   <si>
     <t>J05AB11</t>
@@ -1676,10 +1683,10 @@
     <t>VAL04O</t>
   </si>
   <si>
-    <t>Valcyte 450mg Tab</t>
-  </si>
-  <si>
-    <t>Valganciclovir(Valcyte) 450mg tab</t>
+    <t xml:space="preserve">Valcyte 450mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valganciclovir(Valcyte) 450mg tab</t>
   </si>
   <si>
     <t>J05AB14</t>
@@ -1688,10 +1695,10 @@
     <t>REM02I</t>
   </si>
   <si>
-    <t>Remdesivir (Veklury) 100mg Vial (公費)</t>
-  </si>
-  <si>
-    <t>Remdesivir(Veklury) 100mg Vail (公費)</t>
+    <t xml:space="preserve">Remdesivir (Veklury) 100mg Vial (公費)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remdesivir(Veklury) 100mg Vail (公費)</t>
   </si>
   <si>
     <t>J05AB16</t>
@@ -1700,100 +1707,103 @@
     <t>REM05I</t>
   </si>
   <si>
-    <t>Veklury 100mg Vial  (無健保非本國)</t>
-  </si>
-  <si>
-    <t>Remdesivir(Veklury) 100mg Vail (無健保非本國)</t>
+    <t xml:space="preserve">Veklury 100mg Vial  (無健保非本國)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remdesivir(Veklury) 100mg Vail (無健保非本國)</t>
   </si>
   <si>
     <t>AMO05S</t>
   </si>
   <si>
-    <t>Amoxycillin Sandoz Susp 50mg/mL;100mL</t>
-  </si>
-  <si>
-    <t>Amoxicillin (Amoxycillin Sandoz) Susp 50mg/mL 100mL</t>
+    <t xml:space="preserve">Amoxycillin Sandoz Susp 50mg/mL;100mL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amoxicillin (Amoxycillin Sandoz) Susp 50mg/mL 100mL</t>
   </si>
   <si>
     <t>EXT01I</t>
   </si>
   <si>
-    <t>Extencilline 2.4MUI Vial</t>
-  </si>
-  <si>
-    <t>Benzathine benzylpenicillin (Extencilline) 2.4MUI Vial</t>
+    <t xml:space="preserve">Extencilline 2.4MUI Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benzathine benzylpenicillin (Extencilline) 2.4MUI Vial</t>
   </si>
   <si>
     <t>CEF09I</t>
   </si>
   <si>
-    <t>Cefe 2gm Vial</t>
-  </si>
-  <si>
-    <t>Cefmetazole (Cefe) 2gm Vial</t>
+    <t xml:space="preserve">Cefe 2gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefmetazole (Cefe) 2gm Vial</t>
   </si>
   <si>
     <t>J01DC09</t>
   </si>
   <si>
-    <t>建議量:  1 g to 2 gm q6h@ 2.5gen or 3rd cephas for ESBL@ Ccr 30 to 49: 2 gm q12h@ Ccr 10 to 29: 2 gm qd@ Ccr less 10 or HD: 1 g qd</t>
+    <t xml:space="preserve">建議量:  1 g to 2 gm q6h@ 2.5gen or 3rd cephas for ESBL@ Ccr 30 to 49: 2 gm q12h@ Ccr 10 to 29: 2 gm qd@ Ccr less 10 or HD: 1 g qd</t>
   </si>
   <si>
     <t>PEN11I</t>
   </si>
   <si>
-    <t>Penem 500/500mg Vial</t>
+    <t xml:space="preserve">Penem 500/500mg Vial</t>
   </si>
   <si>
     <t>J01DH51</t>
   </si>
   <si>
-    <t>建議量:  1.25 gm q6h@ imipenem加 cilastatin sodium阻斷 imipenem腎臟代謝@ Ccr 60 to 89: 1 gm q6h@ Ccr 30 to 59: 0.75 gm q6h@ Ccr 15 to 29: 0.5 gm qd@ Ccr less 10 or HD: 0.5 g qd</t>
+    <t xml:space="preserve">建議量:  1.25 gm q6h@ imipenem加 cilastatin sodium阻斷 imipenem腎臟代謝@ Ccr 60 to 89: 1 gm q6h@ Ccr 30 to 59: 0.75 gm q6h@ Ccr 15 to 29: 0.5 gm qd@ Ccr less 10 or HD: 0.5 g qd</t>
   </si>
   <si>
     <t>FET01I</t>
   </si>
   <si>
-    <t>Fetroja 1gm Vial</t>
-  </si>
-  <si>
-    <t>Cefiderocol (Fetroja) 1gm Vial</t>
+    <t xml:space="preserve">Fetroja 1gm Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cefiderocol (Fetroja) 1gm Vial</t>
   </si>
   <si>
     <t>J01DI04</t>
   </si>
   <si>
-    <t>建議量:  2 gm q8h@ Ccr 30 to 59: 1.5 gm q8h@ Ccr 15 to 29: 1 gm q8h@ Ccr less 15 or HD: 0.75 g qd</t>
+    <t xml:space="preserve">建議量:  2 gm q8h@ Ccr 30 to 59: 1.5 gm q8h@ Ccr 15 to 29: 1 gm q8h@ Ccr less 15 or HD: 0.75 g qd</t>
   </si>
   <si>
     <t>BOB01I</t>
   </si>
   <si>
-    <t>Bobimixyn 500KU Vial</t>
-  </si>
-  <si>
-    <t>Polymyxin B (Bobimixyn) 500KU Vial</t>
+    <t xml:space="preserve">Bobimixyn 500KU Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polymyxin B (Bobimixyn) 500KU Vial</t>
   </si>
   <si>
     <t>J01XB02</t>
   </si>
   <si>
+    <t xml:space="preserve">起始劑量（依體重，輸注須超過2小時）:@ 40 kg需2 vial@  50 kg需2.5 vial@  60 kg需3 vial@  70 kg需3.5 vial@  80 kg需4 vial@ 維持劑量:@ 40 kg需1.2 vial@  50 kg需1.5 vial@  60 kg需1.8 vial@  70 kg需2.1 vial@  80 kg需2.4 vial</t>
+  </si>
+  <si>
     <t>DIS02O</t>
   </si>
   <si>
-    <t>Disfect FC 250mg Tab</t>
-  </si>
-  <si>
-    <t>Fusidate (Disfect FC) 250mg Tab</t>
+    <t xml:space="preserve">Disfect FC 250mg Tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusidate (Disfect FC) 250mg Tab</t>
   </si>
   <si>
     <t>ACT10I</t>
   </si>
   <si>
-    <t>Actavir 250mg Vial</t>
-  </si>
-  <si>
-    <t>Acyclovir (Actavir) 250mg Vial</t>
+    <t xml:space="preserve">Actavir 250mg Vial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acyclovir (Actavir) 250mg Vial</t>
   </si>
   <si>
     <t>ATC_CODE</t>
@@ -1826,7 +1836,7 @@
     <t>Minocycline(Cyclin)</t>
   </si>
   <si>
-    <t>100 mg q12h drip 1hr</t>
+    <t xml:space="preserve">100 mg q12h drip 1hr</t>
   </si>
   <si>
     <t>Tigecycline(Tigelin)</t>
@@ -1844,13 +1854,13 @@
     <t>AmoClav</t>
   </si>
   <si>
-    <t>Ccr less 30: 1vial q12h@ Ccr less 10 or HD: 1 vial qd</t>
-  </si>
-  <si>
-    <t>1 gm q8h@ Ccr less 30: 1 gm q12h@ Ccr less 10 or HD: 1 gm qd</t>
-  </si>
-  <si>
-    <t>1# q8h@ Ccr less 30 or HD: clavulanate 排除較amox快易造成治療失敗</t>
+    <t xml:space="preserve">Ccr less 30: 1vial q12h@ Ccr less 10 or HD: 1 vial qd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 gm q8h@ Ccr less 30: 1 gm q12h@ Ccr less 10 or HD: 1 gm qd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1# q8h@ Ccr less 30 or HD: clavulanate 排除較amox快易造成治療失敗</t>
   </si>
   <si>
     <t>Dicloxacillin(Diclocin)</t>
@@ -1865,13 +1875,13 @@
     <t>Subacillin</t>
   </si>
   <si>
-    <t>Ccr less 30: 3 gm q12h@ Ccr less 10 or HD: 3 gm qd</t>
-  </si>
-  <si>
-    <t>40 to 45mg per kg q8h to q12h 以 amoxi 計@ 高劑量: 2倍量頻次不變</t>
-  </si>
-  <si>
-    <t>1 vial q8h@ 小兒: 30 mg per kg q8h 以 amoxi 計@ Ccr less than 30: q12h@ Ccr less than 10, HD or PD: qd</t>
+    <t xml:space="preserve">Ccr less 30: 3 gm q12h@ Ccr less 10 or HD: 3 gm qd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40 to 45mg per kg q8h to q12h 以 amoxi 計@ 高劑量: 2倍量頻次不變</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 vial q8h@ 小兒: 30 mg per kg q8h 以 amoxi 計@ Ccr less than 30: q12h@ Ccr less than 10, HD or PD: qd</t>
   </si>
   <si>
     <t>Sultamicillin</t>
@@ -1886,7 +1896,7 @@
     <t>Cephalexin</t>
   </si>
   <si>
-    <t>Ccr less 30: 1 gm q8h or q12h@ Ccr less 10 or HD: 1 gm qd</t>
+    <t xml:space="preserve">Ccr less 30: 1 gm q8h or q12h@ Ccr less 10 or HD: 1 gm qd</t>
   </si>
   <si>
     <t>Cefazolin(Cefa)</t>
@@ -1913,7 +1923,7 @@
     <t>Cefotaxime(Claforan)</t>
   </si>
   <si>
-    <t>2 gm q6h@ Max: 2 gm q4h@ 小兒: 40 mg per kg q6h to q4h@ Ccr less than 50: 2 gm q8h@ Ccr less than 30: 2 gm q12h@ Ccr less than 10, HD or PD: 1 gm qd</t>
+    <t xml:space="preserve">2 gm q6h@ Max: 2 gm q4h@ 小兒: 40 mg per kg q6h to q4h@ Ccr less than 50: 2 gm q8h@ Ccr less than 30: 2 gm q12h@ Ccr less than 10, HD or PD: 1 gm qd</t>
   </si>
   <si>
     <t>Ceftazidime(Tatumcef)</t>
@@ -1934,7 +1944,7 @@
     <t>Cefoperazone+Sulbactam</t>
   </si>
   <si>
-    <t>無法穿透BBB,膽道濃度高@ 建議量: 4 g q8h@ Ccr less 30: 4 g q12h@ Ccr less 15 or HD: 2 g q12h</t>
+    <t xml:space="preserve">無法穿透BBB,膽道濃度高@ 建議量: 4 g q8h@ Ccr less 30: 4 g q12h@ Ccr less 15 or HD: 2 g q12h</t>
   </si>
   <si>
     <t>Cefepime</t>
@@ -1961,7 +1971,7 @@
     <t>Cotrimoxazol(Baktar)</t>
   </si>
   <si>
-    <t>4 mg TMP per kg q12h@ 預防UTI: 2 mg TMP per kg qd</t>
+    <t xml:space="preserve">4 mg TMP per kg q12h@ 預防UTI: 2 mg TMP per kg qd</t>
   </si>
   <si>
     <t>Erythromycin</t>
@@ -1979,7 +1989,7 @@
     <t>Gentamicin(V-Genta)</t>
   </si>
   <si>
-    <t>1.7 mg per kg q8h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
+    <t xml:space="preserve">1.7 mg per kg q8h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
   </si>
   <si>
     <t>Neomycin</t>
@@ -1988,13 +1998,13 @@
     <t>Amikacin(Acemycin)</t>
   </si>
   <si>
-    <t>7.5 mg per kg q12h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
+    <t xml:space="preserve">7.5 mg per kg q12h@ renal dysfunction: 使用一周後建議監測血中濃度@ 使用二周後必須監測血中濃度</t>
   </si>
   <si>
     <t>Ciprofloxacin(Cinolone)</t>
   </si>
   <si>
-    <t>500 mg to 750 mg qd@ Ccr less than 50: 半劑量 qd@ Ccr less than 20, HD or PD: 半劑量 qod</t>
+    <t xml:space="preserve">500 mg to 750 mg qd@ Ccr less than 50: 半劑量 qd@ Ccr less than 20, HD or PD: 半劑量 qod</t>
   </si>
   <si>
     <t>Moxifloxacin(Avelox)</t>
@@ -2009,7 +2019,7 @@
     <t>Vancomycin</t>
   </si>
   <si>
-    <t>125 mg or 500 mg q6h for 10 days</t>
+    <t xml:space="preserve">125 mg or 500 mg q6h for 10 days</t>
   </si>
   <si>
     <t>Teicoplanin(Targocid)</t>
@@ -2030,34 +2040,34 @@
     <t>Linezolid(Linetero)</t>
   </si>
   <si>
-    <t>600 mg q12h</t>
-  </si>
-  <si>
-    <t>600 mg q12h須空腹</t>
+    <t xml:space="preserve">600 mg q12h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">600 mg q12h須空腹</t>
   </si>
   <si>
     <t>Daptomycin(Cubicin)</t>
   </si>
   <si>
-    <t>組織穿透差不適pneumonia@ endocarditis: 8 to 12 mg per kg qd@ soft tissue: 4 to 6 mg per kg qd@ Ccr less than 30, HD or PD: qod@ DDI: statins following up CPK</t>
+    <t xml:space="preserve">組織穿透差不適pneumonia@ endocarditis: 8 to 12 mg per kg qd@ soft tissue: 4 to 6 mg per kg qd@ Ccr less than 30, HD or PD: qod@ DDI: statins following up CPK</t>
   </si>
   <si>
     <t>Amphotericin</t>
   </si>
   <si>
-    <t>3 to 6 mg per kg once daily</t>
+    <t xml:space="preserve">3 to 6 mg per kg once daily</t>
   </si>
   <si>
     <t>Fluconazole(Diflucan)</t>
   </si>
   <si>
-    <t>200 to 800 mg daily@ Ccr less than 50: 劑量減半@ Ccr less 25: 四分之一劑量@ HD:  洗完正常量</t>
+    <t xml:space="preserve">200 to 800 mg daily@ Ccr less than 50: 劑量減半@ Ccr less 25: 四分之一劑量@ HD:  洗完正常量</t>
   </si>
   <si>
     <t>Itraconazole(Sporanox)</t>
   </si>
   <si>
-    <t>200 mg qd to q12h@ DDI: QTc prolongation@ 禁忌: HF</t>
+    <t xml:space="preserve">200 mg qd to q12h@ DDI: QTc prolongation@ 禁忌: HF</t>
   </si>
   <si>
     <t>Voriconazole</t>
@@ -2069,13 +2079,13 @@
     <t>Flucytosine</t>
   </si>
   <si>
-    <t>25 mg per kg q6h@ Ccr less than 40: q12h@ Ccr less than 20: qd@ Ccr less than 10, HD or PD: qod@ 罕單用經肝臟排泄@ SE: 骨髓抑制@ 禁忌: 孕婦</t>
+    <t xml:space="preserve">25 mg per kg q6h@ Ccr less than 40: q12h@ Ccr less than 20: qd@ Ccr less than 10, HD or PD: qod@ 罕單用經肝臟排泄@ SE: 骨髓抑制@ 禁忌: 孕婦</t>
   </si>
   <si>
     <t>Micafungin(Mycamine)</t>
   </si>
   <si>
-    <t>100 mg to 150 mg qd@ 小兒: 2 to 3 mg per kg qd</t>
+    <t xml:space="preserve">100 mg to 150 mg qd@ 小兒: 2 to 3 mg per kg qd</t>
   </si>
   <si>
     <t>Anidulafungin</t>
@@ -2102,28 +2112,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6">
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="PMingLiu"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="PMingLiu"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color rgb="FFFF0000"/>
+      <sz val="11.000000"/>
+      <color indexed="2"/>
       <name val="PMingLiu"/>
     </font>
     <font>
@@ -2141,76 +2151,358 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -2267,7 +2559,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2293,7 +2585,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2370,7 +2662,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2400,22 +2692,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="9.71"/>
-    <col customWidth="1" min="2" max="2" width="38.86"/>
+    <col customWidth="1" min="1" max="1" width="9.7100000000000009"/>
+    <col customWidth="1" min="2" max="2" width="38.859999999999999"/>
     <col customWidth="1" min="3" max="3" width="16.57"/>
-    <col customWidth="1" min="4" max="4" width="9.29"/>
-    <col customWidth="1" min="5" max="5" width="71.86"/>
-    <col customWidth="1" min="6" max="6" width="10.14"/>
+    <col customWidth="1" min="4" max="4" width="9.2899999999999991"/>
+    <col customWidth="1" min="5" max="5" width="71.859999999999999"/>
+    <col customWidth="1" min="6" max="6" width="10.140000000000001"/>
     <col customWidth="1" min="7" max="26" width="14.57"/>
   </cols>
   <sheetData>
@@ -2488,7 +2782,7 @@
         <v>16</v>
       </c>
       <c r="F4" s="4">
-        <v>11.0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -2572,7 +2866,7 @@
         <v>36</v>
       </c>
       <c r="F9" s="4">
-        <v>16.0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -2592,7 +2886,7 @@
         <v>40</v>
       </c>
       <c r="F10" s="4">
-        <v>83.0</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -2628,7 +2922,7 @@
         <v>48</v>
       </c>
       <c r="F12" s="4">
-        <v>44.0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -2648,7 +2942,7 @@
         <v>52</v>
       </c>
       <c r="F13" s="4">
-        <v>32.0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -2668,7 +2962,7 @@
         <v>57</v>
       </c>
       <c r="F14" s="4">
-        <v>92.0</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -2688,7 +2982,7 @@
         <v>57</v>
       </c>
       <c r="F15" s="4">
-        <v>53.0</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -2708,7 +3002,7 @@
         <v>65</v>
       </c>
       <c r="F16" s="4">
-        <v>55.0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -2728,7 +3022,7 @@
         <v>65</v>
       </c>
       <c r="F17" s="4">
-        <v>24.0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
@@ -2764,7 +3058,7 @@
         <v>75</v>
       </c>
       <c r="F19" s="4">
-        <v>35.0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -2784,7 +3078,7 @@
         <v>79</v>
       </c>
       <c r="F20" s="4">
-        <v>60.0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -2804,7 +3098,7 @@
         <v>79</v>
       </c>
       <c r="F21" s="4">
-        <v>70.0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -2860,7 +3154,7 @@
         <v>93</v>
       </c>
       <c r="F24" s="4">
-        <v>61.0</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -2878,7 +3172,7 @@
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="4">
-        <v>99.0</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -2898,7 +3192,7 @@
         <v>102</v>
       </c>
       <c r="F26" s="4">
-        <v>102.0</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -2918,7 +3212,7 @@
         <v>106</v>
       </c>
       <c r="F27" s="4">
-        <v>49.0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -2970,7 +3264,7 @@
         <v>117</v>
       </c>
       <c r="F30" s="4">
-        <v>3.0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -3024,7 +3318,7 @@
         <v>127</v>
       </c>
       <c r="F33" s="4">
-        <v>91.0</v>
+        <v>91</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
@@ -3044,7 +3338,7 @@
         <v>131</v>
       </c>
       <c r="F34" s="4">
-        <v>90.0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -3064,7 +3358,7 @@
         <v>135</v>
       </c>
       <c r="F35" s="4">
-        <v>20.0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
@@ -3100,7 +3394,7 @@
         <v>143</v>
       </c>
       <c r="F37" s="4">
-        <v>7.0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
@@ -3120,7 +3414,7 @@
         <v>143</v>
       </c>
       <c r="F38" s="4">
-        <v>48.0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -3140,7 +3434,7 @@
         <v>149</v>
       </c>
       <c r="F39" s="4">
-        <v>14.0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -3194,7 +3488,7 @@
         <v>162</v>
       </c>
       <c r="F42" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -3214,7 +3508,7 @@
         <v>167</v>
       </c>
       <c r="F43" s="4">
-        <v>22.0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -3250,7 +3544,7 @@
         <v>173</v>
       </c>
       <c r="F45" s="4">
-        <v>4.0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -3270,7 +3564,7 @@
         <v>178</v>
       </c>
       <c r="F46" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
@@ -3290,7 +3584,7 @@
         <v>183</v>
       </c>
       <c r="F47" s="4">
-        <v>56.0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -3310,7 +3604,7 @@
         <v>188</v>
       </c>
       <c r="F48" s="4">
-        <v>18.0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -3330,7 +3624,7 @@
         <v>188</v>
       </c>
       <c r="F49" s="4">
-        <v>12.0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -3348,7 +3642,7 @@
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="4">
-        <v>30.0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -3368,7 +3662,7 @@
         <v>197</v>
       </c>
       <c r="F51" s="4">
-        <v>40.0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
@@ -3406,7 +3700,7 @@
         <v>197</v>
       </c>
       <c r="F53" s="4">
-        <v>5.0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
@@ -3442,7 +3736,7 @@
         <v>211</v>
       </c>
       <c r="F55" s="4">
-        <v>25.0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
@@ -3462,7 +3756,7 @@
         <v>216</v>
       </c>
       <c r="F56" s="4">
-        <v>6.0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -3482,7 +3776,7 @@
         <v>221</v>
       </c>
       <c r="F57" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -3502,7 +3796,7 @@
         <v>226</v>
       </c>
       <c r="F58" s="4">
-        <v>17.0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
@@ -3522,7 +3816,7 @@
         <v>231</v>
       </c>
       <c r="F59" s="4">
-        <v>21.0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -3542,7 +3836,7 @@
         <v>236</v>
       </c>
       <c r="F60" s="4">
-        <v>26.0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
@@ -3562,7 +3856,7 @@
         <v>241</v>
       </c>
       <c r="F61" s="4">
-        <v>34.0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
@@ -3580,7 +3874,7 @@
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="4">
-        <v>72.0</v>
+        <v>72</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
@@ -3600,7 +3894,7 @@
         <v>249</v>
       </c>
       <c r="F63" s="4">
-        <v>19.0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
@@ -3636,7 +3930,7 @@
         <v>257</v>
       </c>
       <c r="F65" s="4">
-        <v>52.0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
@@ -3656,7 +3950,7 @@
         <v>262</v>
       </c>
       <c r="F66" s="4">
-        <v>98.0</v>
+        <v>98</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
@@ -3692,7 +3986,7 @@
         <v>269</v>
       </c>
       <c r="F68" s="4">
-        <v>71.0</v>
+        <v>71</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
@@ -3712,7 +4006,7 @@
         <v>274</v>
       </c>
       <c r="F69" s="4">
-        <v>31.0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
@@ -3732,7 +4026,7 @@
         <v>279</v>
       </c>
       <c r="F70" s="4">
-        <v>46.0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
@@ -3800,7 +4094,7 @@
         <v>293</v>
       </c>
       <c r="F74" s="4">
-        <v>88.0</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
@@ -3820,7 +4114,7 @@
         <v>298</v>
       </c>
       <c r="F75" s="4">
-        <v>64.0</v>
+        <v>64</v>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
@@ -3840,7 +4134,7 @@
         <v>298</v>
       </c>
       <c r="F76" s="4">
-        <v>75.0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
@@ -3860,7 +4154,7 @@
         <v>293</v>
       </c>
       <c r="F77" s="4">
-        <v>97.0</v>
+        <v>97</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
@@ -3896,7 +4190,7 @@
         <v>311</v>
       </c>
       <c r="F79" s="4">
-        <v>28.0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
@@ -3916,7 +4210,7 @@
         <v>316</v>
       </c>
       <c r="F80" s="4">
-        <v>59.0</v>
+        <v>59</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
@@ -3936,7 +4230,7 @@
         <v>321</v>
       </c>
       <c r="F81" s="4">
-        <v>8.0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
@@ -3956,7 +4250,7 @@
         <v>325</v>
       </c>
       <c r="F82" s="4">
-        <v>76.0</v>
+        <v>76</v>
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
@@ -3976,7 +4270,7 @@
         <v>330</v>
       </c>
       <c r="F83" s="4">
-        <v>57.0</v>
+        <v>57</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
@@ -3996,7 +4290,7 @@
         <v>335</v>
       </c>
       <c r="F84" s="4">
-        <v>37.0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
@@ -4016,7 +4310,7 @@
         <v>340</v>
       </c>
       <c r="F85" s="4">
-        <v>33.0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
@@ -4068,7 +4362,7 @@
         <v>351</v>
       </c>
       <c r="F88" s="4">
-        <v>36.0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
@@ -4088,7 +4382,7 @@
         <v>356</v>
       </c>
       <c r="F89" s="4">
-        <v>15.0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
@@ -4124,7 +4418,7 @@
         <v>364</v>
       </c>
       <c r="F91" s="4">
-        <v>81.0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
@@ -4144,7 +4438,7 @@
         <v>364</v>
       </c>
       <c r="F92" s="4">
-        <v>73.0</v>
+        <v>73</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
@@ -4180,7 +4474,7 @@
         <v>364</v>
       </c>
       <c r="F94" s="4">
-        <v>41.0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
@@ -4200,7 +4494,7 @@
         <v>364</v>
       </c>
       <c r="F95" s="4">
-        <v>84.0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
@@ -4220,7 +4514,7 @@
         <v>382</v>
       </c>
       <c r="F96" s="4">
-        <v>101.0</v>
+        <v>101</v>
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
@@ -4240,7 +4534,7 @@
         <v>387</v>
       </c>
       <c r="F97" s="4">
-        <v>80.0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
@@ -4260,7 +4554,7 @@
         <v>387</v>
       </c>
       <c r="F98" s="4">
-        <v>50.0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
@@ -4296,7 +4590,7 @@
         <v>397</v>
       </c>
       <c r="F100" s="4">
-        <v>38.0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1">
@@ -4316,7 +4610,7 @@
         <v>402</v>
       </c>
       <c r="F101" s="4">
-        <v>54.0</v>
+        <v>54</v>
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1">
@@ -4336,7 +4630,7 @@
         <v>407</v>
       </c>
       <c r="F102" s="4">
-        <v>67.0</v>
+        <v>67</v>
       </c>
     </row>
     <row r="103" ht="15.75" customHeight="1">
@@ -4356,7 +4650,7 @@
         <v>407</v>
       </c>
       <c r="F103" s="4">
-        <v>9.0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1">
@@ -4376,7 +4670,7 @@
         <v>415</v>
       </c>
       <c r="F104" s="4">
-        <v>27.0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="105" ht="15.75" customHeight="1">
@@ -4396,7 +4690,7 @@
         <v>420</v>
       </c>
       <c r="F105" s="4">
-        <v>62.0</v>
+        <v>62</v>
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
@@ -4464,7 +4758,7 @@
         <v>433</v>
       </c>
       <c r="F109" s="4">
-        <v>13.0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="110" ht="15.75" customHeight="1">
@@ -4484,7 +4778,7 @@
         <v>433</v>
       </c>
       <c r="F110" s="4">
-        <v>51.0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="111" ht="15.75" customHeight="1">
@@ -4522,7 +4816,7 @@
         <v>444</v>
       </c>
       <c r="F112" s="4">
-        <v>85.0</v>
+        <v>85</v>
       </c>
     </row>
     <row r="113" ht="15.75" customHeight="1">
@@ -4540,7 +4834,7 @@
       </c>
       <c r="E113" s="3"/>
       <c r="F113" s="4">
-        <v>95.0</v>
+        <v>95</v>
       </c>
     </row>
     <row r="114" ht="15.75" customHeight="1">
@@ -4560,7 +4854,7 @@
         <v>452</v>
       </c>
       <c r="F114" s="4">
-        <v>93.0</v>
+        <v>93</v>
       </c>
     </row>
     <row r="115" ht="15.75" customHeight="1">
@@ -4580,7 +4874,7 @@
         <v>457</v>
       </c>
       <c r="F115" s="4">
-        <v>45.0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="116" ht="15.75" customHeight="1">
@@ -4600,7 +4894,7 @@
         <v>452</v>
       </c>
       <c r="F116" s="4">
-        <v>89.0</v>
+        <v>89</v>
       </c>
     </row>
     <row r="117" ht="15.75" customHeight="1">
@@ -4620,7 +4914,7 @@
         <v>465</v>
       </c>
       <c r="F117" s="4">
-        <v>23.0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="118" ht="15.75" customHeight="1">
@@ -4640,7 +4934,7 @@
         <v>470</v>
       </c>
       <c r="F118" s="4">
-        <v>63.0</v>
+        <v>63</v>
       </c>
     </row>
     <row r="119" ht="15.75" customHeight="1">
@@ -4660,7 +4954,7 @@
         <v>470</v>
       </c>
       <c r="F119" s="4">
-        <v>79.0</v>
+        <v>79</v>
       </c>
     </row>
     <row r="120" ht="15.75" customHeight="1">
@@ -4698,7 +4992,7 @@
         <v>482</v>
       </c>
       <c r="F121" s="4">
-        <v>47.0</v>
+        <v>47</v>
       </c>
     </row>
     <row r="122" ht="15.75" customHeight="1">
@@ -4718,7 +5012,7 @@
         <v>482</v>
       </c>
       <c r="F122" s="4">
-        <v>42.0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="123" ht="15.75" customHeight="1">
@@ -4738,7 +5032,7 @@
         <v>482</v>
       </c>
       <c r="F123" s="4">
-        <v>82.0</v>
+        <v>82</v>
       </c>
     </row>
     <row r="124" ht="15.75" customHeight="1">
@@ -4758,7 +5052,7 @@
         <v>493</v>
       </c>
       <c r="F124" s="4">
-        <v>100.0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="125" ht="15.75" customHeight="1">
@@ -4778,7 +5072,7 @@
         <v>498</v>
       </c>
       <c r="F125" s="4">
-        <v>78.0</v>
+        <v>78</v>
       </c>
     </row>
     <row r="126" ht="15.75" customHeight="1">
@@ -4798,7 +5092,7 @@
         <v>503</v>
       </c>
       <c r="F126" s="4">
-        <v>87.0</v>
+        <v>87</v>
       </c>
     </row>
     <row r="127" ht="15.75" customHeight="1">
@@ -4818,7 +5112,7 @@
         <v>508</v>
       </c>
       <c r="F127" s="4">
-        <v>86.0</v>
+        <v>86</v>
       </c>
     </row>
     <row r="128" ht="15.75" customHeight="1">
@@ -4838,7 +5132,7 @@
         <v>513</v>
       </c>
       <c r="F128" s="4">
-        <v>69.0</v>
+        <v>69</v>
       </c>
     </row>
     <row r="129" ht="15.75" customHeight="1">
@@ -4858,7 +5152,7 @@
         <v>518</v>
       </c>
       <c r="F129" s="4">
-        <v>68.0</v>
+        <v>68</v>
       </c>
     </row>
     <row r="130" ht="15.75" customHeight="1">
@@ -4878,7 +5172,7 @@
         <v>523</v>
       </c>
       <c r="F130" s="4">
-        <v>39.0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="131" ht="15.75" customHeight="1">
@@ -4898,7 +5192,7 @@
         <v>528</v>
       </c>
       <c r="F131" s="4">
-        <v>58.0</v>
+        <v>58</v>
       </c>
     </row>
     <row r="132" ht="15.75" customHeight="1">
@@ -4918,7 +5212,7 @@
         <v>533</v>
       </c>
       <c r="F132" s="4">
-        <v>96.0</v>
+        <v>96</v>
       </c>
     </row>
     <row r="133" ht="15.75" customHeight="1">
@@ -4938,7 +5232,7 @@
         <v>533</v>
       </c>
       <c r="F133" s="4">
-        <v>43.0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="134" ht="15.75" customHeight="1">
@@ -4956,7 +5250,7 @@
       </c>
       <c r="E134" s="3"/>
       <c r="F134" s="4">
-        <v>65.0</v>
+        <v>65</v>
       </c>
     </row>
     <row r="135" ht="15.75" customHeight="1">
@@ -4974,7 +5268,7 @@
       </c>
       <c r="E135" s="3"/>
       <c r="F135" s="4">
-        <v>66.0</v>
+        <v>66</v>
       </c>
     </row>
     <row r="136" ht="15.75" customHeight="1">
@@ -4992,7 +5286,7 @@
       </c>
       <c r="E136" s="3"/>
       <c r="F136" s="4">
-        <v>94.0</v>
+        <v>94</v>
       </c>
     </row>
     <row r="137" ht="15.75" customHeight="1">
@@ -5010,7 +5304,7 @@
       </c>
       <c r="E137" s="3"/>
       <c r="F137" s="4">
-        <v>77.0</v>
+        <v>77</v>
       </c>
     </row>
     <row r="138" ht="15.75" customHeight="1">
@@ -5028,7 +5322,7 @@
       </c>
       <c r="E138" s="3"/>
       <c r="F138" s="4">
-        <v>74.0</v>
+        <v>74</v>
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1">
@@ -5046,7 +5340,7 @@
       </c>
       <c r="E139" s="3"/>
       <c r="F139" s="4">
-        <v>29.0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="140" ht="15.75" customHeight="1">
@@ -5064,7 +5358,7 @@
       </c>
       <c r="E140" s="3"/>
       <c r="F140" s="4">
-        <v>103.0</v>
+        <v>103</v>
       </c>
     </row>
     <row r="141" ht="15.75" customHeight="1">
@@ -5154,7 +5448,7 @@
       </c>
       <c r="F145" s="7"/>
     </row>
-    <row r="146" ht="15.75" customHeight="1">
+    <row r="146" ht="17.25" customHeight="1">
       <c r="A146" s="6" t="s">
         <v>583</v>
       </c>
@@ -5167,17 +5461,20 @@
       <c r="D146" s="9" t="s">
         <v>586</v>
       </c>
+      <c r="E146" s="9" t="s">
+        <v>587</v>
+      </c>
       <c r="F146" s="7"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="8" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C147" s="6" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>419</v>
@@ -5189,13 +5486,13 @@
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="8" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C148" s="6" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>532</v>
@@ -6443,30 +6740,31 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="$A$1:$F$148"/>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="14.86"/>
+    <col customWidth="1" min="1" max="1" width="14.859999999999999"/>
     <col customWidth="1" min="2" max="2" width="25.57"/>
-    <col customWidth="1" min="3" max="3" width="156.57"/>
-    <col customWidth="1" min="4" max="6" width="9.14"/>
+    <col customWidth="1" min="3" max="3" width="156.56999999999999"/>
+    <col customWidth="1" min="4" max="6" width="9.1400000000000006"/>
     <col customWidth="1" min="7" max="26" width="14.57"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -6480,7 +6778,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C2" s="3"/>
     </row>
@@ -6489,7 +6787,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>16</v>
@@ -6500,7 +6798,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -6509,7 +6807,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -6518,7 +6816,7 @@
         <v>28</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C6" s="3"/>
     </row>
@@ -6527,10 +6825,10 @@
         <v>35</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
     </row>
     <row r="8" ht="17.25" customHeight="1">
@@ -6538,7 +6836,7 @@
         <v>39</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>40</v>
@@ -6549,10 +6847,10 @@
         <v>44</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="10" ht="17.25" customHeight="1">
@@ -6560,7 +6858,7 @@
         <v>56</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>57</v>
@@ -6568,10 +6866,10 @@
     </row>
     <row r="11" ht="17.25" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -6580,7 +6878,7 @@
         <v>64</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>65</v>
@@ -6591,10 +6889,10 @@
         <v>74</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -6605,7 +6903,7 @@
         <v>81</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="15" ht="17.25" customHeight="1">
@@ -6627,7 +6925,7 @@
         <v>133</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="17" ht="17.25" customHeight="1">
@@ -6635,7 +6933,7 @@
         <v>92</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>93</v>
@@ -6646,7 +6944,7 @@
         <v>97</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C18" s="3"/>
     </row>
@@ -6655,7 +6953,7 @@
         <v>101</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>102</v>
@@ -6666,7 +6964,7 @@
         <v>105</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>106</v>
@@ -6677,7 +6975,7 @@
         <v>110</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C21" s="3"/>
     </row>
@@ -6686,10 +6984,10 @@
         <v>116</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
     </row>
     <row r="23" ht="17.25" customHeight="1">
@@ -6700,7 +6998,7 @@
         <v>125</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
     </row>
     <row r="24" ht="17.25" customHeight="1">
@@ -6711,7 +7009,7 @@
         <v>130</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="25" ht="17.25" customHeight="1">
@@ -6722,7 +7020,7 @@
         <v>133</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="26" ht="17.25" customHeight="1">
@@ -6730,7 +7028,7 @@
         <v>139</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C26" s="3"/>
     </row>
@@ -6739,10 +7037,10 @@
         <v>142</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
     </row>
     <row r="28" ht="17.25" customHeight="1">
@@ -6750,10 +7048,10 @@
         <v>148</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="29" ht="17.25" customHeight="1">
@@ -6761,7 +7059,7 @@
         <v>153</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>154</v>
@@ -6772,10 +7070,10 @@
         <v>158</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
     <row r="31" ht="17.25" customHeight="1">
@@ -6794,10 +7092,10 @@
         <v>166</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="33" ht="17.25" customHeight="1">
@@ -6808,7 +7106,7 @@
         <v>172</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
     <row r="34" ht="17.25" customHeight="1">
@@ -6816,10 +7114,10 @@
         <v>177</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
     </row>
     <row r="35" ht="17.25" customHeight="1">
@@ -6827,10 +7125,10 @@
         <v>182</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="36" ht="17.25" customHeight="1">
@@ -6838,10 +7136,10 @@
         <v>187</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="37" ht="17.25" customHeight="1">
@@ -6849,10 +7147,10 @@
         <v>196</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
     </row>
     <row r="38" ht="17.25" customHeight="1">
@@ -6860,7 +7158,7 @@
         <v>207</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>211</v>
@@ -6871,10 +7169,10 @@
         <v>215</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
     </row>
     <row r="40" ht="17.25" customHeight="1">
@@ -6882,7 +7180,7 @@
         <v>220</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>221</v>
@@ -6893,7 +7191,7 @@
         <v>225</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>226</v>
@@ -6904,10 +7202,10 @@
         <v>230</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="43" ht="17.25" customHeight="1">
@@ -6937,7 +7235,7 @@
         <v>235</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>236</v>
@@ -6948,7 +7246,7 @@
         <v>240</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>241</v>
@@ -6959,7 +7257,7 @@
         <v>244</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C47" s="3"/>
     </row>
@@ -6968,7 +7266,7 @@
         <v>248</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>249</v>
@@ -6993,7 +7291,7 @@
         <v>260</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
     </row>
     <row r="51" ht="17.25" customHeight="1">
@@ -7001,7 +7299,7 @@
         <v>266</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C51" s="3"/>
     </row>
@@ -7010,7 +7308,7 @@
         <v>273</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>274</v>
@@ -7032,7 +7330,7 @@
         <v>297</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>298</v>
@@ -7054,7 +7352,7 @@
         <v>307</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>335</v>
@@ -7076,10 +7374,10 @@
         <v>320</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="59" ht="17.25" customHeight="1">
@@ -7087,7 +7385,7 @@
         <v>324</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>325</v>
@@ -7098,10 +7396,10 @@
         <v>329</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="61" ht="17.25" customHeight="1">
@@ -7109,7 +7407,7 @@
         <v>334</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>335</v>
@@ -7145,7 +7443,7 @@
         <v>354</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
     </row>
     <row r="65" ht="17.25" customHeight="1">
@@ -7153,7 +7451,7 @@
         <v>363</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>364</v>
@@ -7175,7 +7473,7 @@
         <v>381</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>382</v>
@@ -7186,7 +7484,7 @@
         <v>386</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C68" s="3"/>
     </row>
@@ -7195,7 +7493,7 @@
         <v>393</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>397</v>
@@ -7209,7 +7507,7 @@
         <v>400</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
     </row>
     <row r="71" ht="17.25" customHeight="1">
@@ -7217,7 +7515,7 @@
         <v>406</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>407</v>
@@ -7228,7 +7526,7 @@
         <v>414</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>415</v>
@@ -7239,7 +7537,7 @@
         <v>419</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>420</v>
@@ -7250,7 +7548,7 @@
         <v>427</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C74" s="3"/>
     </row>
@@ -7259,7 +7557,7 @@
         <v>443</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C75" s="3"/>
     </row>
@@ -7268,10 +7566,10 @@
         <v>456</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
     </row>
     <row r="77" ht="17.25" customHeight="1">
@@ -7282,7 +7580,7 @@
         <v>460</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
     </row>
     <row r="78" ht="17.25" customHeight="1">
@@ -7290,10 +7588,10 @@
         <v>464</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="79" ht="17.25" customHeight="1">
@@ -7301,10 +7599,10 @@
         <v>469</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
     </row>
     <row r="80" ht="17.25" customHeight="1">
@@ -7312,10 +7610,10 @@
         <v>481</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
     </row>
     <row r="81" ht="17.25" customHeight="1">
@@ -7323,10 +7621,10 @@
         <v>492</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
     </row>
     <row r="82" ht="17.25" customHeight="1">
@@ -7334,7 +7632,7 @@
         <v>497</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>498</v>
@@ -7356,7 +7654,7 @@
         <v>507</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>508</v>
@@ -7367,10 +7665,10 @@
         <v>512</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
     </row>
     <row r="86" ht="17.25" customHeight="1">
@@ -7378,10 +7676,10 @@
         <v>517</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
     </row>
     <row r="87" ht="17.25" customHeight="1">
@@ -7389,7 +7687,7 @@
         <v>522</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>523</v>
@@ -7400,7 +7698,7 @@
         <v>527</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>528</v>
@@ -7422,7 +7720,7 @@
         <v>540</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="C90" s="3"/>
     </row>
@@ -7431,7 +7729,7 @@
         <v>547</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C91" s="3"/>
     </row>
@@ -7440,7 +7738,7 @@
         <v>551</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C92" s="3"/>
     </row>
@@ -7449,7 +7747,7 @@
         <v>555</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C93" s="3"/>
     </row>
@@ -7458,7 +7756,7 @@
         <v>559</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C94" s="3"/>
     </row>
@@ -8372,21 +8670,22 @@
     <row r="1002" ht="15.75" customHeight="1"/>
     <row r="1003" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="8.86"/>
+    <col customWidth="1" min="1" max="26" width="8.8599999999999994"/>
   </cols>
   <sheetData>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -9370,9 +9669,9 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>